<commit_message>
Actualizar vigas de pisos superiores
</commit_message>
<xml_diff>
--- a/nodos_modelo_manual.xlsx
+++ b/nodos_modelo_manual.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H145"/>
+  <dimension ref="A1:H153"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4529,7 +4529,7 @@
         <v>900022</v>
       </c>
       <c r="B129" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C129" t="inlineStr">
         <is>
@@ -4537,13 +4537,13 @@
         </is>
       </c>
       <c r="D129" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="E129" t="n">
         <v>-4.12</v>
       </c>
       <c r="F129" t="n">
-        <v>11.88</v>
+        <v>19.8</v>
       </c>
       <c r="G129" t="inlineStr">
         <is>
@@ -4561,7 +4561,7 @@
         <v>900023</v>
       </c>
       <c r="B130" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C130" t="inlineStr">
         <is>
@@ -4569,13 +4569,13 @@
         </is>
       </c>
       <c r="D130" t="n">
-        <v>17.49</v>
+        <v>30</v>
       </c>
       <c r="E130" t="n">
         <v>-4.12</v>
       </c>
       <c r="F130" t="n">
-        <v>11.88</v>
+        <v>19.8</v>
       </c>
       <c r="G130" t="inlineStr">
         <is>
@@ -4601,10 +4601,10 @@
         </is>
       </c>
       <c r="D131" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="E131" t="n">
-        <v>0</v>
+        <v>-4.12</v>
       </c>
       <c r="F131" t="n">
         <v>11.88</v>
@@ -4633,10 +4633,10 @@
         </is>
       </c>
       <c r="D132" t="n">
-        <v>15</v>
+        <v>17.49</v>
       </c>
       <c r="E132" t="n">
-        <v>15.84</v>
+        <v>-4.12</v>
       </c>
       <c r="F132" t="n">
         <v>11.88</v>
@@ -4665,10 +4665,10 @@
         </is>
       </c>
       <c r="D133" t="n">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="E133" t="n">
-        <v>15.84</v>
+        <v>0</v>
       </c>
       <c r="F133" t="n">
         <v>11.88</v>
@@ -4697,10 +4697,10 @@
         </is>
       </c>
       <c r="D134" t="n">
-        <v>17.49</v>
+        <v>15</v>
       </c>
       <c r="E134" t="n">
-        <v>0</v>
+        <v>15.84</v>
       </c>
       <c r="F134" t="n">
         <v>11.88</v>
@@ -4729,10 +4729,10 @@
         </is>
       </c>
       <c r="D135" t="n">
-        <v>17.49</v>
+        <v>25</v>
       </c>
       <c r="E135" t="n">
-        <v>7.25</v>
+        <v>15.84</v>
       </c>
       <c r="F135" t="n">
         <v>11.88</v>
@@ -4761,7 +4761,7 @@
         </is>
       </c>
       <c r="D136" t="n">
-        <v>35</v>
+        <v>17.49</v>
       </c>
       <c r="E136" t="n">
         <v>0</v>
@@ -4793,10 +4793,10 @@
         </is>
       </c>
       <c r="D137" t="n">
-        <v>35</v>
+        <v>17.49</v>
       </c>
       <c r="E137" t="n">
-        <v>15.84</v>
+        <v>7.25</v>
       </c>
       <c r="F137" t="n">
         <v>11.88</v>
@@ -4817,7 +4817,7 @@
         <v>900031</v>
       </c>
       <c r="B138" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C138" t="inlineStr">
         <is>
@@ -4825,13 +4825,13 @@
         </is>
       </c>
       <c r="D138" t="n">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="E138" t="n">
         <v>0</v>
       </c>
       <c r="F138" t="n">
-        <v>15.84</v>
+        <v>11.88</v>
       </c>
       <c r="G138" t="inlineStr">
         <is>
@@ -4849,7 +4849,7 @@
         <v>900032</v>
       </c>
       <c r="B139" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C139" t="inlineStr">
         <is>
@@ -4857,13 +4857,13 @@
         </is>
       </c>
       <c r="D139" t="n">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="E139" t="n">
         <v>15.84</v>
       </c>
       <c r="F139" t="n">
-        <v>15.84</v>
+        <v>11.88</v>
       </c>
       <c r="G139" t="inlineStr">
         <is>
@@ -4889,7 +4889,7 @@
         </is>
       </c>
       <c r="D140" t="n">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="E140" t="n">
         <v>0</v>
@@ -4921,7 +4921,7 @@
         </is>
       </c>
       <c r="D141" t="n">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="E141" t="n">
         <v>15.84</v>
@@ -4953,7 +4953,7 @@
         </is>
       </c>
       <c r="D142" t="n">
-        <v>17.49</v>
+        <v>25</v>
       </c>
       <c r="E142" t="n">
         <v>0</v>
@@ -4985,10 +4985,10 @@
         </is>
       </c>
       <c r="D143" t="n">
-        <v>17.49</v>
+        <v>25</v>
       </c>
       <c r="E143" t="n">
-        <v>7.25</v>
+        <v>15.84</v>
       </c>
       <c r="F143" t="n">
         <v>15.84</v>
@@ -5063,6 +5063,262 @@
         </is>
       </c>
       <c r="H145" t="inlineStr">
+        <is>
+          <t>MANUAL_BEAM_NODE</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="n">
+        <v>900039</v>
+      </c>
+      <c r="B146" t="n">
+        <v>5</v>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>BEAM_MANUAL</t>
+        </is>
+      </c>
+      <c r="D146" t="n">
+        <v>47.55</v>
+      </c>
+      <c r="E146" t="n">
+        <v>0</v>
+      </c>
+      <c r="F146" t="n">
+        <v>19.8</v>
+      </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>Libre</t>
+        </is>
+      </c>
+      <c r="H146" t="inlineStr">
+        <is>
+          <t>MANUAL_BEAM_NODE</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="n">
+        <v>900040</v>
+      </c>
+      <c r="B147" t="n">
+        <v>5</v>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>BEAM_MANUAL</t>
+        </is>
+      </c>
+      <c r="D147" t="n">
+        <v>47.55</v>
+      </c>
+      <c r="E147" t="n">
+        <v>15.84</v>
+      </c>
+      <c r="F147" t="n">
+        <v>19.8</v>
+      </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>Libre</t>
+        </is>
+      </c>
+      <c r="H147" t="inlineStr">
+        <is>
+          <t>MANUAL_BEAM_NODE</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="n">
+        <v>900041</v>
+      </c>
+      <c r="B148" t="n">
+        <v>5</v>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>BEAM_MANUAL</t>
+        </is>
+      </c>
+      <c r="D148" t="n">
+        <v>15</v>
+      </c>
+      <c r="E148" t="n">
+        <v>0</v>
+      </c>
+      <c r="F148" t="n">
+        <v>19.8</v>
+      </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>Libre</t>
+        </is>
+      </c>
+      <c r="H148" t="inlineStr">
+        <is>
+          <t>MANUAL_BEAM_NODE</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="n">
+        <v>900042</v>
+      </c>
+      <c r="B149" t="n">
+        <v>5</v>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>BEAM_MANUAL</t>
+        </is>
+      </c>
+      <c r="D149" t="n">
+        <v>15</v>
+      </c>
+      <c r="E149" t="n">
+        <v>15.84</v>
+      </c>
+      <c r="F149" t="n">
+        <v>19.8</v>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>Libre</t>
+        </is>
+      </c>
+      <c r="H149" t="inlineStr">
+        <is>
+          <t>MANUAL_BEAM_NODE</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="n">
+        <v>900043</v>
+      </c>
+      <c r="B150" t="n">
+        <v>5</v>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>BEAM_MANUAL</t>
+        </is>
+      </c>
+      <c r="D150" t="n">
+        <v>25</v>
+      </c>
+      <c r="E150" t="n">
+        <v>0</v>
+      </c>
+      <c r="F150" t="n">
+        <v>19.8</v>
+      </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>Libre</t>
+        </is>
+      </c>
+      <c r="H150" t="inlineStr">
+        <is>
+          <t>MANUAL_BEAM_NODE</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="n">
+        <v>900044</v>
+      </c>
+      <c r="B151" t="n">
+        <v>5</v>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>BEAM_MANUAL</t>
+        </is>
+      </c>
+      <c r="D151" t="n">
+        <v>25</v>
+      </c>
+      <c r="E151" t="n">
+        <v>15.84</v>
+      </c>
+      <c r="F151" t="n">
+        <v>19.8</v>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>Libre</t>
+        </is>
+      </c>
+      <c r="H151" t="inlineStr">
+        <is>
+          <t>MANUAL_BEAM_NODE</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="n">
+        <v>900045</v>
+      </c>
+      <c r="B152" t="n">
+        <v>5</v>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>BEAM_MANUAL</t>
+        </is>
+      </c>
+      <c r="D152" t="n">
+        <v>35</v>
+      </c>
+      <c r="E152" t="n">
+        <v>0</v>
+      </c>
+      <c r="F152" t="n">
+        <v>19.8</v>
+      </c>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>Libre</t>
+        </is>
+      </c>
+      <c r="H152" t="inlineStr">
+        <is>
+          <t>MANUAL_BEAM_NODE</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="n">
+        <v>900046</v>
+      </c>
+      <c r="B153" t="n">
+        <v>5</v>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>BEAM_MANUAL</t>
+        </is>
+      </c>
+      <c r="D153" t="n">
+        <v>35</v>
+      </c>
+      <c r="E153" t="n">
+        <v>15.84</v>
+      </c>
+      <c r="F153" t="n">
+        <v>19.8</v>
+      </c>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>Libre</t>
+        </is>
+      </c>
+      <c r="H153" t="inlineStr">
         <is>
           <t>MANUAL_BEAM_NODE</t>
         </is>
@@ -5079,7 +5335,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E186"/>
+  <dimension ref="A1:E173"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7723,10 +7979,10 @@
         </is>
       </c>
       <c r="C126" t="n">
-        <v>300001</v>
+        <v>900022</v>
       </c>
       <c r="D126" t="n">
-        <v>300451</v>
+        <v>900023</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -7744,10 +8000,10 @@
         </is>
       </c>
       <c r="C127" t="n">
-        <v>301001</v>
+        <v>300001</v>
       </c>
       <c r="D127" t="n">
-        <v>301451</v>
+        <v>300451</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -7765,10 +8021,10 @@
         </is>
       </c>
       <c r="C128" t="n">
-        <v>302001</v>
+        <v>301001</v>
       </c>
       <c r="D128" t="n">
-        <v>302451</v>
+        <v>301451</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -7786,10 +8042,10 @@
         </is>
       </c>
       <c r="C129" t="n">
-        <v>900022</v>
+        <v>302001</v>
       </c>
       <c r="D129" t="n">
-        <v>900023</v>
+        <v>302451</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -7803,14 +8059,14 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>BEAM_Y</t>
+          <t>BEAM_X</t>
         </is>
       </c>
       <c r="C130" t="n">
-        <v>300001</v>
+        <v>900024</v>
       </c>
       <c r="D130" t="n">
-        <v>302001</v>
+        <v>900025</v>
       </c>
       <c r="E130" t="inlineStr">
         <is>
@@ -7828,10 +8084,10 @@
         </is>
       </c>
       <c r="C131" t="n">
-        <v>300101</v>
+        <v>300001</v>
       </c>
       <c r="D131" t="n">
-        <v>302101</v>
+        <v>302001</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -7849,10 +8105,10 @@
         </is>
       </c>
       <c r="C132" t="n">
-        <v>300201</v>
+        <v>300101</v>
       </c>
       <c r="D132" t="n">
-        <v>302201</v>
+        <v>302101</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -7870,10 +8126,10 @@
         </is>
       </c>
       <c r="C133" t="n">
-        <v>300301</v>
+        <v>300201</v>
       </c>
       <c r="D133" t="n">
-        <v>302301</v>
+        <v>302201</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -7891,10 +8147,10 @@
         </is>
       </c>
       <c r="C134" t="n">
-        <v>300401</v>
+        <v>300301</v>
       </c>
       <c r="D134" t="n">
-        <v>302401</v>
+        <v>302301</v>
       </c>
       <c r="E134" t="inlineStr">
         <is>
@@ -7912,10 +8168,10 @@
         </is>
       </c>
       <c r="C135" t="n">
-        <v>300451</v>
+        <v>300401</v>
       </c>
       <c r="D135" t="n">
-        <v>302451</v>
+        <v>302401</v>
       </c>
       <c r="E135" t="inlineStr">
         <is>
@@ -7933,10 +8189,10 @@
         </is>
       </c>
       <c r="C136" t="n">
-        <v>900022</v>
+        <v>300451</v>
       </c>
       <c r="D136" t="n">
-        <v>300101</v>
+        <v>302451</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -7957,7 +8213,7 @@
         <v>900024</v>
       </c>
       <c r="D137" t="n">
-        <v>900025</v>
+        <v>300101</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -7975,10 +8231,10 @@
         </is>
       </c>
       <c r="C138" t="n">
-        <v>900011</v>
+        <v>900026</v>
       </c>
       <c r="D138" t="n">
-        <v>900026</v>
+        <v>900027</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
@@ -7996,7 +8252,7 @@
         </is>
       </c>
       <c r="C139" t="n">
-        <v>900027</v>
+        <v>900011</v>
       </c>
       <c r="D139" t="n">
         <v>900028</v>
@@ -8017,10 +8273,10 @@
         </is>
       </c>
       <c r="C140" t="n">
-        <v>900023</v>
+        <v>900029</v>
       </c>
       <c r="D140" t="n">
-        <v>900027</v>
+        <v>900030</v>
       </c>
       <c r="E140" t="inlineStr">
         <is>
@@ -8038,10 +8294,10 @@
         </is>
       </c>
       <c r="C141" t="n">
+        <v>900025</v>
+      </c>
+      <c r="D141" t="n">
         <v>900029</v>
-      </c>
-      <c r="D141" t="n">
-        <v>900030</v>
       </c>
       <c r="E141" t="inlineStr">
         <is>
@@ -8055,14 +8311,14 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>BEAM_X</t>
+          <t>BEAM_Y</t>
         </is>
       </c>
       <c r="C142" t="n">
-        <v>400001</v>
+        <v>900031</v>
       </c>
       <c r="D142" t="n">
-        <v>400451</v>
+        <v>900032</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
@@ -8080,10 +8336,10 @@
         </is>
       </c>
       <c r="C143" t="n">
-        <v>401001</v>
+        <v>400001</v>
       </c>
       <c r="D143" t="n">
-        <v>401451</v>
+        <v>400451</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -8101,10 +8357,10 @@
         </is>
       </c>
       <c r="C144" t="n">
-        <v>402001</v>
+        <v>401001</v>
       </c>
       <c r="D144" t="n">
-        <v>402451</v>
+        <v>401451</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
@@ -8118,14 +8374,14 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>BEAM_Y</t>
+          <t>BEAM_X</t>
         </is>
       </c>
       <c r="C145" t="n">
-        <v>400001</v>
+        <v>402001</v>
       </c>
       <c r="D145" t="n">
-        <v>402001</v>
+        <v>402451</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
@@ -8143,10 +8399,10 @@
         </is>
       </c>
       <c r="C146" t="n">
-        <v>400101</v>
+        <v>400001</v>
       </c>
       <c r="D146" t="n">
-        <v>402101</v>
+        <v>402001</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
@@ -8164,10 +8420,10 @@
         </is>
       </c>
       <c r="C147" t="n">
-        <v>400201</v>
+        <v>400101</v>
       </c>
       <c r="D147" t="n">
-        <v>402201</v>
+        <v>402101</v>
       </c>
       <c r="E147" t="inlineStr">
         <is>
@@ -8185,10 +8441,10 @@
         </is>
       </c>
       <c r="C148" t="n">
-        <v>400301</v>
+        <v>400201</v>
       </c>
       <c r="D148" t="n">
-        <v>402301</v>
+        <v>402201</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
@@ -8206,10 +8462,10 @@
         </is>
       </c>
       <c r="C149" t="n">
-        <v>400401</v>
+        <v>400301</v>
       </c>
       <c r="D149" t="n">
-        <v>402401</v>
+        <v>402301</v>
       </c>
       <c r="E149" t="inlineStr">
         <is>
@@ -8227,10 +8483,10 @@
         </is>
       </c>
       <c r="C150" t="n">
-        <v>400451</v>
+        <v>400401</v>
       </c>
       <c r="D150" t="n">
-        <v>402451</v>
+        <v>402401</v>
       </c>
       <c r="E150" t="inlineStr">
         <is>
@@ -8248,10 +8504,10 @@
         </is>
       </c>
       <c r="C151" t="n">
-        <v>900031</v>
+        <v>400451</v>
       </c>
       <c r="D151" t="n">
-        <v>900032</v>
+        <v>402451</v>
       </c>
       <c r="E151" t="inlineStr">
         <is>
@@ -8328,18 +8584,18 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>BEAM_X</t>
+          <t>BEAM_Y</t>
         </is>
       </c>
       <c r="C155" t="n">
-        <v>500001</v>
+        <v>500201</v>
       </c>
       <c r="D155" t="n">
-        <v>500101</v>
+        <v>900022</v>
       </c>
       <c r="E155" t="inlineStr">
         <is>
-          <t>PROVISIONAL_BEAM</t>
+          <t>MANUAL</t>
         </is>
       </c>
     </row>
@@ -8349,18 +8605,18 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>BEAM_X</t>
+          <t>BEAM_Y</t>
         </is>
       </c>
       <c r="C156" t="n">
-        <v>500101</v>
+        <v>500301</v>
       </c>
       <c r="D156" t="n">
-        <v>500201</v>
+        <v>900023</v>
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>PROVISIONAL_BEAM</t>
+          <t>MANUAL</t>
         </is>
       </c>
     </row>
@@ -8374,14 +8630,14 @@
         </is>
       </c>
       <c r="C157" t="n">
-        <v>500201</v>
+        <v>502451</v>
       </c>
       <c r="D157" t="n">
-        <v>500301</v>
+        <v>502501</v>
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>PROVISIONAL_BEAM</t>
+          <t>MANUAL</t>
         </is>
       </c>
     </row>
@@ -8395,14 +8651,14 @@
         </is>
       </c>
       <c r="C158" t="n">
-        <v>500301</v>
+        <v>501451</v>
       </c>
       <c r="D158" t="n">
-        <v>500401</v>
+        <v>501501</v>
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>PROVISIONAL_BEAM</t>
+          <t>MANUAL</t>
         </is>
       </c>
     </row>
@@ -8416,14 +8672,14 @@
         </is>
       </c>
       <c r="C159" t="n">
-        <v>500401</v>
+        <v>500451</v>
       </c>
       <c r="D159" t="n">
-        <v>500451</v>
+        <v>500501</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>PROVISIONAL_BEAM</t>
+          <t>MANUAL</t>
         </is>
       </c>
     </row>
@@ -8433,18 +8689,18 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>BEAM_X</t>
+          <t>BEAM_40x60</t>
         </is>
       </c>
       <c r="C160" t="n">
-        <v>500451</v>
+        <v>900039</v>
       </c>
       <c r="D160" t="n">
-        <v>500501</v>
+        <v>900040</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t>PROVISIONAL_BEAM</t>
+          <t>MANUAL</t>
         </is>
       </c>
     </row>
@@ -8454,18 +8710,18 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>BEAM_X</t>
+          <t>BEAM_Y</t>
         </is>
       </c>
       <c r="C161" t="n">
-        <v>501001</v>
+        <v>500501</v>
       </c>
       <c r="D161" t="n">
-        <v>501101</v>
+        <v>502501</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
-          <t>PROVISIONAL_BEAM</t>
+          <t>MANUAL</t>
         </is>
       </c>
     </row>
@@ -8479,14 +8735,14 @@
         </is>
       </c>
       <c r="C162" t="n">
-        <v>501101</v>
+        <v>500001</v>
       </c>
       <c r="D162" t="n">
-        <v>501201</v>
+        <v>500451</v>
       </c>
       <c r="E162" t="inlineStr">
         <is>
-          <t>PROVISIONAL_BEAM</t>
+          <t>MANUAL</t>
         </is>
       </c>
     </row>
@@ -8500,14 +8756,14 @@
         </is>
       </c>
       <c r="C163" t="n">
-        <v>501201</v>
+        <v>501001</v>
       </c>
       <c r="D163" t="n">
-        <v>501301</v>
+        <v>501451</v>
       </c>
       <c r="E163" t="inlineStr">
         <is>
-          <t>PROVISIONAL_BEAM</t>
+          <t>MANUAL</t>
         </is>
       </c>
     </row>
@@ -8521,14 +8777,14 @@
         </is>
       </c>
       <c r="C164" t="n">
-        <v>501301</v>
+        <v>502001</v>
       </c>
       <c r="D164" t="n">
-        <v>501401</v>
+        <v>502451</v>
       </c>
       <c r="E164" t="inlineStr">
         <is>
-          <t>PROVISIONAL_BEAM</t>
+          <t>MANUAL</t>
         </is>
       </c>
     </row>
@@ -8538,18 +8794,18 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>BEAM_X</t>
+          <t>BEAM_Y</t>
         </is>
       </c>
       <c r="C165" t="n">
-        <v>501401</v>
+        <v>500001</v>
       </c>
       <c r="D165" t="n">
-        <v>501451</v>
+        <v>502001</v>
       </c>
       <c r="E165" t="inlineStr">
         <is>
-          <t>PROVISIONAL_BEAM</t>
+          <t>MANUAL</t>
         </is>
       </c>
     </row>
@@ -8559,18 +8815,18 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>BEAM_X</t>
+          <t>BEAM_Y</t>
         </is>
       </c>
       <c r="C166" t="n">
-        <v>501451</v>
+        <v>500101</v>
       </c>
       <c r="D166" t="n">
-        <v>501501</v>
+        <v>502101</v>
       </c>
       <c r="E166" t="inlineStr">
         <is>
-          <t>PROVISIONAL_BEAM</t>
+          <t>MANUAL</t>
         </is>
       </c>
     </row>
@@ -8580,18 +8836,18 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>BEAM_X</t>
+          <t>BEAM_Y</t>
         </is>
       </c>
       <c r="C167" t="n">
-        <v>502001</v>
+        <v>500201</v>
       </c>
       <c r="D167" t="n">
-        <v>502101</v>
+        <v>502201</v>
       </c>
       <c r="E167" t="inlineStr">
         <is>
-          <t>PROVISIONAL_BEAM</t>
+          <t>MANUAL</t>
         </is>
       </c>
     </row>
@@ -8601,18 +8857,18 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>BEAM_X</t>
+          <t>BEAM_Y</t>
         </is>
       </c>
       <c r="C168" t="n">
-        <v>502101</v>
+        <v>500301</v>
       </c>
       <c r="D168" t="n">
-        <v>502201</v>
+        <v>502301</v>
       </c>
       <c r="E168" t="inlineStr">
         <is>
-          <t>PROVISIONAL_BEAM</t>
+          <t>MANUAL</t>
         </is>
       </c>
     </row>
@@ -8622,18 +8878,18 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>BEAM_X</t>
+          <t>BEAM_Y</t>
         </is>
       </c>
       <c r="C169" t="n">
-        <v>502201</v>
+        <v>500401</v>
       </c>
       <c r="D169" t="n">
-        <v>502301</v>
+        <v>502401</v>
       </c>
       <c r="E169" t="inlineStr">
         <is>
-          <t>PROVISIONAL_BEAM</t>
+          <t>MANUAL</t>
         </is>
       </c>
     </row>
@@ -8643,18 +8899,18 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>BEAM_X</t>
+          <t>BEAM_Y</t>
         </is>
       </c>
       <c r="C170" t="n">
-        <v>502301</v>
+        <v>500451</v>
       </c>
       <c r="D170" t="n">
-        <v>502401</v>
+        <v>502451</v>
       </c>
       <c r="E170" t="inlineStr">
         <is>
-          <t>PROVISIONAL_BEAM</t>
+          <t>MANUAL</t>
         </is>
       </c>
     </row>
@@ -8664,18 +8920,18 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>BEAM_X</t>
+          <t>BEAM_Y</t>
         </is>
       </c>
       <c r="C171" t="n">
-        <v>502401</v>
+        <v>900041</v>
       </c>
       <c r="D171" t="n">
-        <v>502451</v>
+        <v>900042</v>
       </c>
       <c r="E171" t="inlineStr">
         <is>
-          <t>PROVISIONAL_BEAM</t>
+          <t>MANUAL</t>
         </is>
       </c>
     </row>
@@ -8685,18 +8941,18 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>BEAM_X</t>
+          <t>BEAM_Y</t>
         </is>
       </c>
       <c r="C172" t="n">
-        <v>502451</v>
+        <v>900043</v>
       </c>
       <c r="D172" t="n">
-        <v>502501</v>
+        <v>900044</v>
       </c>
       <c r="E172" t="inlineStr">
         <is>
-          <t>PROVISIONAL_BEAM</t>
+          <t>MANUAL</t>
         </is>
       </c>
     </row>
@@ -8710,287 +8966,14 @@
         </is>
       </c>
       <c r="C173" t="n">
-        <v>500001</v>
+        <v>900045</v>
       </c>
       <c r="D173" t="n">
-        <v>501001</v>
+        <v>900046</v>
       </c>
       <c r="E173" t="inlineStr">
         <is>
-          <t>PROVISIONAL_BEAM</t>
-        </is>
-      </c>
-    </row>
-    <row r="174">
-      <c r="A174" t="n">
-        <v>173</v>
-      </c>
-      <c r="B174" t="inlineStr">
-        <is>
-          <t>BEAM_Y</t>
-        </is>
-      </c>
-      <c r="C174" t="n">
-        <v>501001</v>
-      </c>
-      <c r="D174" t="n">
-        <v>502001</v>
-      </c>
-      <c r="E174" t="inlineStr">
-        <is>
-          <t>PROVISIONAL_BEAM</t>
-        </is>
-      </c>
-    </row>
-    <row r="175">
-      <c r="A175" t="n">
-        <v>174</v>
-      </c>
-      <c r="B175" t="inlineStr">
-        <is>
-          <t>BEAM_Y</t>
-        </is>
-      </c>
-      <c r="C175" t="n">
-        <v>500101</v>
-      </c>
-      <c r="D175" t="n">
-        <v>501101</v>
-      </c>
-      <c r="E175" t="inlineStr">
-        <is>
-          <t>PROVISIONAL_BEAM</t>
-        </is>
-      </c>
-    </row>
-    <row r="176">
-      <c r="A176" t="n">
-        <v>175</v>
-      </c>
-      <c r="B176" t="inlineStr">
-        <is>
-          <t>BEAM_Y</t>
-        </is>
-      </c>
-      <c r="C176" t="n">
-        <v>501101</v>
-      </c>
-      <c r="D176" t="n">
-        <v>502101</v>
-      </c>
-      <c r="E176" t="inlineStr">
-        <is>
-          <t>PROVISIONAL_BEAM</t>
-        </is>
-      </c>
-    </row>
-    <row r="177">
-      <c r="A177" t="n">
-        <v>176</v>
-      </c>
-      <c r="B177" t="inlineStr">
-        <is>
-          <t>BEAM_Y</t>
-        </is>
-      </c>
-      <c r="C177" t="n">
-        <v>500201</v>
-      </c>
-      <c r="D177" t="n">
-        <v>501201</v>
-      </c>
-      <c r="E177" t="inlineStr">
-        <is>
-          <t>PROVISIONAL_BEAM</t>
-        </is>
-      </c>
-    </row>
-    <row r="178">
-      <c r="A178" t="n">
-        <v>177</v>
-      </c>
-      <c r="B178" t="inlineStr">
-        <is>
-          <t>BEAM_Y</t>
-        </is>
-      </c>
-      <c r="C178" t="n">
-        <v>501201</v>
-      </c>
-      <c r="D178" t="n">
-        <v>502201</v>
-      </c>
-      <c r="E178" t="inlineStr">
-        <is>
-          <t>PROVISIONAL_BEAM</t>
-        </is>
-      </c>
-    </row>
-    <row r="179">
-      <c r="A179" t="n">
-        <v>178</v>
-      </c>
-      <c r="B179" t="inlineStr">
-        <is>
-          <t>BEAM_Y</t>
-        </is>
-      </c>
-      <c r="C179" t="n">
-        <v>500301</v>
-      </c>
-      <c r="D179" t="n">
-        <v>501301</v>
-      </c>
-      <c r="E179" t="inlineStr">
-        <is>
-          <t>PROVISIONAL_BEAM</t>
-        </is>
-      </c>
-    </row>
-    <row r="180">
-      <c r="A180" t="n">
-        <v>179</v>
-      </c>
-      <c r="B180" t="inlineStr">
-        <is>
-          <t>BEAM_Y</t>
-        </is>
-      </c>
-      <c r="C180" t="n">
-        <v>501301</v>
-      </c>
-      <c r="D180" t="n">
-        <v>502301</v>
-      </c>
-      <c r="E180" t="inlineStr">
-        <is>
-          <t>PROVISIONAL_BEAM</t>
-        </is>
-      </c>
-    </row>
-    <row r="181">
-      <c r="A181" t="n">
-        <v>180</v>
-      </c>
-      <c r="B181" t="inlineStr">
-        <is>
-          <t>BEAM_Y</t>
-        </is>
-      </c>
-      <c r="C181" t="n">
-        <v>500401</v>
-      </c>
-      <c r="D181" t="n">
-        <v>501401</v>
-      </c>
-      <c r="E181" t="inlineStr">
-        <is>
-          <t>PROVISIONAL_BEAM</t>
-        </is>
-      </c>
-    </row>
-    <row r="182">
-      <c r="A182" t="n">
-        <v>181</v>
-      </c>
-      <c r="B182" t="inlineStr">
-        <is>
-          <t>BEAM_Y</t>
-        </is>
-      </c>
-      <c r="C182" t="n">
-        <v>501401</v>
-      </c>
-      <c r="D182" t="n">
-        <v>502401</v>
-      </c>
-      <c r="E182" t="inlineStr">
-        <is>
-          <t>PROVISIONAL_BEAM</t>
-        </is>
-      </c>
-    </row>
-    <row r="183">
-      <c r="A183" t="n">
-        <v>182</v>
-      </c>
-      <c r="B183" t="inlineStr">
-        <is>
-          <t>BEAM_Y</t>
-        </is>
-      </c>
-      <c r="C183" t="n">
-        <v>500451</v>
-      </c>
-      <c r="D183" t="n">
-        <v>501451</v>
-      </c>
-      <c r="E183" t="inlineStr">
-        <is>
-          <t>PROVISIONAL_BEAM</t>
-        </is>
-      </c>
-    </row>
-    <row r="184">
-      <c r="A184" t="n">
-        <v>183</v>
-      </c>
-      <c r="B184" t="inlineStr">
-        <is>
-          <t>BEAM_Y</t>
-        </is>
-      </c>
-      <c r="C184" t="n">
-        <v>501451</v>
-      </c>
-      <c r="D184" t="n">
-        <v>502451</v>
-      </c>
-      <c r="E184" t="inlineStr">
-        <is>
-          <t>PROVISIONAL_BEAM</t>
-        </is>
-      </c>
-    </row>
-    <row r="185">
-      <c r="A185" t="n">
-        <v>184</v>
-      </c>
-      <c r="B185" t="inlineStr">
-        <is>
-          <t>BEAM_Y</t>
-        </is>
-      </c>
-      <c r="C185" t="n">
-        <v>500501</v>
-      </c>
-      <c r="D185" t="n">
-        <v>501501</v>
-      </c>
-      <c r="E185" t="inlineStr">
-        <is>
-          <t>PROVISIONAL_BEAM</t>
-        </is>
-      </c>
-    </row>
-    <row r="186">
-      <c r="A186" t="n">
-        <v>185</v>
-      </c>
-      <c r="B186" t="inlineStr">
-        <is>
-          <t>BEAM_Y</t>
-        </is>
-      </c>
-      <c r="C186" t="n">
-        <v>501501</v>
-      </c>
-      <c r="D186" t="n">
-        <v>502501</v>
-      </c>
-      <c r="E186" t="inlineStr">
-        <is>
-          <t>PROVISIONAL_BEAM</t>
+          <t>MANUAL</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Agregar losas estructurales y ajustar su nivel
</commit_message>
<xml_diff>
--- a/nodos_modelo_manual.xlsx
+++ b/nodos_modelo_manual.xlsx
@@ -9,7 +9,8 @@
   <sheets>
     <sheet name="Nodos_Manual" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Elementos" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Supuestos" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Losas" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Supuestos" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -415,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H278"/>
+  <dimension ref="A1:H288"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6609,7 +6610,7 @@
         <v>900039</v>
       </c>
       <c r="B194" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C194" t="inlineStr">
         <is>
@@ -6617,13 +6618,13 @@
         </is>
       </c>
       <c r="D194" t="n">
-        <v>-32.05</v>
+        <v>15</v>
       </c>
       <c r="E194" t="n">
         <v>0</v>
       </c>
       <c r="F194" t="n">
-        <v>7.92</v>
+        <v>19.8</v>
       </c>
       <c r="G194" t="inlineStr">
         <is>
@@ -6641,7 +6642,7 @@
         <v>900040</v>
       </c>
       <c r="B195" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C195" t="inlineStr">
         <is>
@@ -6649,13 +6650,13 @@
         </is>
       </c>
       <c r="D195" t="n">
-        <v>-0.25</v>
+        <v>15</v>
       </c>
       <c r="E195" t="n">
-        <v>0</v>
+        <v>16.15</v>
       </c>
       <c r="F195" t="n">
-        <v>7.92</v>
+        <v>19.8</v>
       </c>
       <c r="G195" t="inlineStr">
         <is>
@@ -6673,7 +6674,7 @@
         <v>900041</v>
       </c>
       <c r="B196" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C196" t="inlineStr">
         <is>
@@ -6681,13 +6682,13 @@
         </is>
       </c>
       <c r="D196" t="n">
-        <v>-0.25</v>
+        <v>25</v>
       </c>
       <c r="E196" t="n">
-        <v>7.25</v>
+        <v>0</v>
       </c>
       <c r="F196" t="n">
-        <v>7.92</v>
+        <v>19.8</v>
       </c>
       <c r="G196" t="inlineStr">
         <is>
@@ -6705,7 +6706,7 @@
         <v>900042</v>
       </c>
       <c r="B197" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C197" t="inlineStr">
         <is>
@@ -6713,13 +6714,13 @@
         </is>
       </c>
       <c r="D197" t="n">
-        <v>-32.05</v>
+        <v>25</v>
       </c>
       <c r="E197" t="n">
         <v>16.15</v>
       </c>
       <c r="F197" t="n">
-        <v>7.92</v>
+        <v>19.8</v>
       </c>
       <c r="G197" t="inlineStr">
         <is>
@@ -6737,7 +6738,7 @@
         <v>900043</v>
       </c>
       <c r="B198" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C198" t="inlineStr">
         <is>
@@ -6745,13 +6746,13 @@
         </is>
       </c>
       <c r="D198" t="n">
-        <v>-0.25</v>
+        <v>35</v>
       </c>
       <c r="E198" t="n">
-        <v>16.15</v>
+        <v>0</v>
       </c>
       <c r="F198" t="n">
-        <v>7.92</v>
+        <v>19.8</v>
       </c>
       <c r="G198" t="inlineStr">
         <is>
@@ -6769,7 +6770,7 @@
         <v>900044</v>
       </c>
       <c r="B199" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C199" t="inlineStr">
         <is>
@@ -6777,13 +6778,13 @@
         </is>
       </c>
       <c r="D199" t="n">
-        <v>-32.05</v>
+        <v>35</v>
       </c>
       <c r="E199" t="n">
-        <v>11.885</v>
+        <v>16.15</v>
       </c>
       <c r="F199" t="n">
-        <v>7.92</v>
+        <v>19.8</v>
       </c>
       <c r="G199" t="inlineStr">
         <is>
@@ -6801,7 +6802,7 @@
         <v>900045</v>
       </c>
       <c r="B200" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C200" t="inlineStr">
         <is>
@@ -6809,13 +6810,13 @@
         </is>
       </c>
       <c r="D200" t="n">
-        <v>-24.55</v>
+        <v>47.55</v>
       </c>
       <c r="E200" t="n">
-        <v>11.885</v>
+        <v>0</v>
       </c>
       <c r="F200" t="n">
-        <v>7.92</v>
+        <v>19.8</v>
       </c>
       <c r="G200" t="inlineStr">
         <is>
@@ -6833,7 +6834,7 @@
         <v>900046</v>
       </c>
       <c r="B201" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C201" t="inlineStr">
         <is>
@@ -6841,13 +6842,13 @@
         </is>
       </c>
       <c r="D201" t="n">
-        <v>-32.05</v>
+        <v>47.55</v>
       </c>
       <c r="E201" t="n">
-        <v>4.265</v>
+        <v>16.15</v>
       </c>
       <c r="F201" t="n">
-        <v>7.92</v>
+        <v>19.8</v>
       </c>
       <c r="G201" t="inlineStr">
         <is>
@@ -6865,7 +6866,7 @@
         <v>900047</v>
       </c>
       <c r="B202" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C202" t="inlineStr">
         <is>
@@ -6873,13 +6874,13 @@
         </is>
       </c>
       <c r="D202" t="n">
-        <v>-24.55</v>
+        <v>20</v>
       </c>
       <c r="E202" t="n">
-        <v>4.265</v>
+        <v>-4.12</v>
       </c>
       <c r="F202" t="n">
-        <v>7.92</v>
+        <v>19.8</v>
       </c>
       <c r="G202" t="inlineStr">
         <is>
@@ -6897,7 +6898,7 @@
         <v>900048</v>
       </c>
       <c r="B203" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C203" t="inlineStr">
         <is>
@@ -6905,13 +6906,13 @@
         </is>
       </c>
       <c r="D203" t="n">
-        <v>-28.3</v>
+        <v>30</v>
       </c>
       <c r="E203" t="n">
-        <v>0</v>
+        <v>-4.12</v>
       </c>
       <c r="F203" t="n">
-        <v>7.92</v>
+        <v>19.8</v>
       </c>
       <c r="G203" t="inlineStr">
         <is>
@@ -6937,10 +6938,10 @@
         </is>
       </c>
       <c r="D204" t="n">
-        <v>-28.3</v>
+        <v>-32.05</v>
       </c>
       <c r="E204" t="n">
-        <v>16.15</v>
+        <v>0</v>
       </c>
       <c r="F204" t="n">
         <v>7.92</v>
@@ -6969,7 +6970,7 @@
         </is>
       </c>
       <c r="D205" t="n">
-        <v>-24.55</v>
+        <v>-0.25</v>
       </c>
       <c r="E205" t="n">
         <v>0</v>
@@ -7001,10 +7002,10 @@
         </is>
       </c>
       <c r="D206" t="n">
-        <v>-24.55</v>
+        <v>-0.25</v>
       </c>
       <c r="E206" t="n">
-        <v>16.15</v>
+        <v>7.25</v>
       </c>
       <c r="F206" t="n">
         <v>7.92</v>
@@ -7033,10 +7034,10 @@
         </is>
       </c>
       <c r="D207" t="n">
-        <v>-15.8</v>
+        <v>-32.05</v>
       </c>
       <c r="E207" t="n">
-        <v>0</v>
+        <v>16.15</v>
       </c>
       <c r="F207" t="n">
         <v>7.92</v>
@@ -7065,7 +7066,7 @@
         </is>
       </c>
       <c r="D208" t="n">
-        <v>-15.8</v>
+        <v>-0.25</v>
       </c>
       <c r="E208" t="n">
         <v>16.15</v>
@@ -7097,10 +7098,10 @@
         </is>
       </c>
       <c r="D209" t="n">
-        <v>-5.8</v>
+        <v>-32.05</v>
       </c>
       <c r="E209" t="n">
-        <v>0</v>
+        <v>11.885</v>
       </c>
       <c r="F209" t="n">
         <v>7.92</v>
@@ -7129,10 +7130,10 @@
         </is>
       </c>
       <c r="D210" t="n">
-        <v>-5.8</v>
+        <v>-24.55</v>
       </c>
       <c r="E210" t="n">
-        <v>16.15</v>
+        <v>11.885</v>
       </c>
       <c r="F210" t="n">
         <v>7.92</v>
@@ -7153,7 +7154,7 @@
         <v>900056</v>
       </c>
       <c r="B211" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C211" t="inlineStr">
         <is>
@@ -7164,10 +7165,10 @@
         <v>-32.05</v>
       </c>
       <c r="E211" t="n">
-        <v>0</v>
+        <v>4.265</v>
       </c>
       <c r="F211" t="n">
-        <v>11.88</v>
+        <v>7.92</v>
       </c>
       <c r="G211" t="inlineStr">
         <is>
@@ -7185,7 +7186,7 @@
         <v>900057</v>
       </c>
       <c r="B212" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C212" t="inlineStr">
         <is>
@@ -7193,13 +7194,13 @@
         </is>
       </c>
       <c r="D212" t="n">
-        <v>-0.25</v>
+        <v>-24.55</v>
       </c>
       <c r="E212" t="n">
-        <v>0</v>
+        <v>4.265</v>
       </c>
       <c r="F212" t="n">
-        <v>11.88</v>
+        <v>7.92</v>
       </c>
       <c r="G212" t="inlineStr">
         <is>
@@ -7217,7 +7218,7 @@
         <v>900058</v>
       </c>
       <c r="B213" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C213" t="inlineStr">
         <is>
@@ -7225,13 +7226,13 @@
         </is>
       </c>
       <c r="D213" t="n">
-        <v>-0.25</v>
+        <v>-28.3</v>
       </c>
       <c r="E213" t="n">
-        <v>7.25</v>
+        <v>0</v>
       </c>
       <c r="F213" t="n">
-        <v>11.88</v>
+        <v>7.92</v>
       </c>
       <c r="G213" t="inlineStr">
         <is>
@@ -7249,7 +7250,7 @@
         <v>900059</v>
       </c>
       <c r="B214" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C214" t="inlineStr">
         <is>
@@ -7257,13 +7258,13 @@
         </is>
       </c>
       <c r="D214" t="n">
-        <v>-32.05</v>
+        <v>-28.3</v>
       </c>
       <c r="E214" t="n">
         <v>16.15</v>
       </c>
       <c r="F214" t="n">
-        <v>11.88</v>
+        <v>7.92</v>
       </c>
       <c r="G214" t="inlineStr">
         <is>
@@ -7281,7 +7282,7 @@
         <v>900060</v>
       </c>
       <c r="B215" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C215" t="inlineStr">
         <is>
@@ -7289,13 +7290,13 @@
         </is>
       </c>
       <c r="D215" t="n">
-        <v>-0.25</v>
+        <v>-24.55</v>
       </c>
       <c r="E215" t="n">
-        <v>16.15</v>
+        <v>0</v>
       </c>
       <c r="F215" t="n">
-        <v>11.88</v>
+        <v>7.92</v>
       </c>
       <c r="G215" t="inlineStr">
         <is>
@@ -7313,7 +7314,7 @@
         <v>900061</v>
       </c>
       <c r="B216" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C216" t="inlineStr">
         <is>
@@ -7321,13 +7322,13 @@
         </is>
       </c>
       <c r="D216" t="n">
-        <v>-32.05</v>
+        <v>-24.55</v>
       </c>
       <c r="E216" t="n">
-        <v>11.885</v>
+        <v>16.15</v>
       </c>
       <c r="F216" t="n">
-        <v>11.88</v>
+        <v>7.92</v>
       </c>
       <c r="G216" t="inlineStr">
         <is>
@@ -7345,7 +7346,7 @@
         <v>900062</v>
       </c>
       <c r="B217" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C217" t="inlineStr">
         <is>
@@ -7353,13 +7354,13 @@
         </is>
       </c>
       <c r="D217" t="n">
-        <v>-24.55</v>
+        <v>-15.8</v>
       </c>
       <c r="E217" t="n">
-        <v>11.885</v>
+        <v>0</v>
       </c>
       <c r="F217" t="n">
-        <v>11.88</v>
+        <v>7.92</v>
       </c>
       <c r="G217" t="inlineStr">
         <is>
@@ -7377,7 +7378,7 @@
         <v>900063</v>
       </c>
       <c r="B218" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C218" t="inlineStr">
         <is>
@@ -7385,13 +7386,13 @@
         </is>
       </c>
       <c r="D218" t="n">
-        <v>-32.05</v>
+        <v>-15.8</v>
       </c>
       <c r="E218" t="n">
-        <v>4.265</v>
+        <v>16.15</v>
       </c>
       <c r="F218" t="n">
-        <v>11.88</v>
+        <v>7.92</v>
       </c>
       <c r="G218" t="inlineStr">
         <is>
@@ -7409,7 +7410,7 @@
         <v>900064</v>
       </c>
       <c r="B219" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C219" t="inlineStr">
         <is>
@@ -7417,13 +7418,13 @@
         </is>
       </c>
       <c r="D219" t="n">
-        <v>-24.55</v>
+        <v>-5.8</v>
       </c>
       <c r="E219" t="n">
-        <v>4.265</v>
+        <v>0</v>
       </c>
       <c r="F219" t="n">
-        <v>11.88</v>
+        <v>7.92</v>
       </c>
       <c r="G219" t="inlineStr">
         <is>
@@ -7441,7 +7442,7 @@
         <v>900065</v>
       </c>
       <c r="B220" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C220" t="inlineStr">
         <is>
@@ -7449,13 +7450,13 @@
         </is>
       </c>
       <c r="D220" t="n">
-        <v>-28.3</v>
+        <v>-5.8</v>
       </c>
       <c r="E220" t="n">
-        <v>0</v>
+        <v>16.15</v>
       </c>
       <c r="F220" t="n">
-        <v>11.88</v>
+        <v>7.92</v>
       </c>
       <c r="G220" t="inlineStr">
         <is>
@@ -7481,10 +7482,10 @@
         </is>
       </c>
       <c r="D221" t="n">
-        <v>-28.3</v>
+        <v>-32.05</v>
       </c>
       <c r="E221" t="n">
-        <v>16.15</v>
+        <v>0</v>
       </c>
       <c r="F221" t="n">
         <v>11.88</v>
@@ -7513,7 +7514,7 @@
         </is>
       </c>
       <c r="D222" t="n">
-        <v>-24.55</v>
+        <v>-0.25</v>
       </c>
       <c r="E222" t="n">
         <v>0</v>
@@ -7545,10 +7546,10 @@
         </is>
       </c>
       <c r="D223" t="n">
-        <v>-24.55</v>
+        <v>-0.25</v>
       </c>
       <c r="E223" t="n">
-        <v>16.15</v>
+        <v>7.25</v>
       </c>
       <c r="F223" t="n">
         <v>11.88</v>
@@ -7577,10 +7578,10 @@
         </is>
       </c>
       <c r="D224" t="n">
-        <v>-15.8</v>
+        <v>-32.05</v>
       </c>
       <c r="E224" t="n">
-        <v>0</v>
+        <v>16.15</v>
       </c>
       <c r="F224" t="n">
         <v>11.88</v>
@@ -7609,7 +7610,7 @@
         </is>
       </c>
       <c r="D225" t="n">
-        <v>-15.8</v>
+        <v>-0.25</v>
       </c>
       <c r="E225" t="n">
         <v>16.15</v>
@@ -7641,10 +7642,10 @@
         </is>
       </c>
       <c r="D226" t="n">
-        <v>-5.8</v>
+        <v>-32.05</v>
       </c>
       <c r="E226" t="n">
-        <v>0</v>
+        <v>11.885</v>
       </c>
       <c r="F226" t="n">
         <v>11.88</v>
@@ -7673,10 +7674,10 @@
         </is>
       </c>
       <c r="D227" t="n">
-        <v>-5.8</v>
+        <v>-24.55</v>
       </c>
       <c r="E227" t="n">
-        <v>16.15</v>
+        <v>11.885</v>
       </c>
       <c r="F227" t="n">
         <v>11.88</v>
@@ -7697,7 +7698,7 @@
         <v>900073</v>
       </c>
       <c r="B228" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C228" t="inlineStr">
         <is>
@@ -7708,10 +7709,10 @@
         <v>-32.05</v>
       </c>
       <c r="E228" t="n">
-        <v>0</v>
+        <v>4.265</v>
       </c>
       <c r="F228" t="n">
-        <v>15.84</v>
+        <v>11.88</v>
       </c>
       <c r="G228" t="inlineStr">
         <is>
@@ -7729,7 +7730,7 @@
         <v>900074</v>
       </c>
       <c r="B229" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C229" t="inlineStr">
         <is>
@@ -7737,13 +7738,13 @@
         </is>
       </c>
       <c r="D229" t="n">
-        <v>-0.25</v>
+        <v>-24.55</v>
       </c>
       <c r="E229" t="n">
-        <v>0</v>
+        <v>4.265</v>
       </c>
       <c r="F229" t="n">
-        <v>15.84</v>
+        <v>11.88</v>
       </c>
       <c r="G229" t="inlineStr">
         <is>
@@ -7761,7 +7762,7 @@
         <v>900075</v>
       </c>
       <c r="B230" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C230" t="inlineStr">
         <is>
@@ -7769,13 +7770,13 @@
         </is>
       </c>
       <c r="D230" t="n">
-        <v>-0.25</v>
+        <v>-28.3</v>
       </c>
       <c r="E230" t="n">
-        <v>7.25</v>
+        <v>0</v>
       </c>
       <c r="F230" t="n">
-        <v>15.84</v>
+        <v>11.88</v>
       </c>
       <c r="G230" t="inlineStr">
         <is>
@@ -7793,7 +7794,7 @@
         <v>900076</v>
       </c>
       <c r="B231" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C231" t="inlineStr">
         <is>
@@ -7801,13 +7802,13 @@
         </is>
       </c>
       <c r="D231" t="n">
-        <v>-32.05</v>
+        <v>-28.3</v>
       </c>
       <c r="E231" t="n">
         <v>16.15</v>
       </c>
       <c r="F231" t="n">
-        <v>15.84</v>
+        <v>11.88</v>
       </c>
       <c r="G231" t="inlineStr">
         <is>
@@ -7825,7 +7826,7 @@
         <v>900077</v>
       </c>
       <c r="B232" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C232" t="inlineStr">
         <is>
@@ -7833,13 +7834,13 @@
         </is>
       </c>
       <c r="D232" t="n">
-        <v>-0.25</v>
+        <v>-24.55</v>
       </c>
       <c r="E232" t="n">
-        <v>16.15</v>
+        <v>0</v>
       </c>
       <c r="F232" t="n">
-        <v>15.84</v>
+        <v>11.88</v>
       </c>
       <c r="G232" t="inlineStr">
         <is>
@@ -7857,7 +7858,7 @@
         <v>900078</v>
       </c>
       <c r="B233" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C233" t="inlineStr">
         <is>
@@ -7865,13 +7866,13 @@
         </is>
       </c>
       <c r="D233" t="n">
-        <v>-32.05</v>
+        <v>-24.55</v>
       </c>
       <c r="E233" t="n">
-        <v>11.885</v>
+        <v>16.15</v>
       </c>
       <c r="F233" t="n">
-        <v>15.84</v>
+        <v>11.88</v>
       </c>
       <c r="G233" t="inlineStr">
         <is>
@@ -7889,7 +7890,7 @@
         <v>900079</v>
       </c>
       <c r="B234" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C234" t="inlineStr">
         <is>
@@ -7897,13 +7898,13 @@
         </is>
       </c>
       <c r="D234" t="n">
-        <v>-24.55</v>
+        <v>-15.8</v>
       </c>
       <c r="E234" t="n">
-        <v>11.885</v>
+        <v>0</v>
       </c>
       <c r="F234" t="n">
-        <v>15.84</v>
+        <v>11.88</v>
       </c>
       <c r="G234" t="inlineStr">
         <is>
@@ -7921,7 +7922,7 @@
         <v>900080</v>
       </c>
       <c r="B235" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C235" t="inlineStr">
         <is>
@@ -7929,13 +7930,13 @@
         </is>
       </c>
       <c r="D235" t="n">
-        <v>-32.05</v>
+        <v>-15.8</v>
       </c>
       <c r="E235" t="n">
-        <v>4.265</v>
+        <v>16.15</v>
       </c>
       <c r="F235" t="n">
-        <v>15.84</v>
+        <v>11.88</v>
       </c>
       <c r="G235" t="inlineStr">
         <is>
@@ -7953,7 +7954,7 @@
         <v>900081</v>
       </c>
       <c r="B236" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C236" t="inlineStr">
         <is>
@@ -7961,13 +7962,13 @@
         </is>
       </c>
       <c r="D236" t="n">
-        <v>-24.55</v>
+        <v>-5.8</v>
       </c>
       <c r="E236" t="n">
-        <v>4.265</v>
+        <v>0</v>
       </c>
       <c r="F236" t="n">
-        <v>15.84</v>
+        <v>11.88</v>
       </c>
       <c r="G236" t="inlineStr">
         <is>
@@ -7985,7 +7986,7 @@
         <v>900082</v>
       </c>
       <c r="B237" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C237" t="inlineStr">
         <is>
@@ -7993,13 +7994,13 @@
         </is>
       </c>
       <c r="D237" t="n">
-        <v>-28.3</v>
+        <v>-5.8</v>
       </c>
       <c r="E237" t="n">
-        <v>0</v>
+        <v>16.15</v>
       </c>
       <c r="F237" t="n">
-        <v>15.84</v>
+        <v>11.88</v>
       </c>
       <c r="G237" t="inlineStr">
         <is>
@@ -8025,10 +8026,10 @@
         </is>
       </c>
       <c r="D238" t="n">
-        <v>-28.3</v>
+        <v>-32.05</v>
       </c>
       <c r="E238" t="n">
-        <v>16.15</v>
+        <v>0</v>
       </c>
       <c r="F238" t="n">
         <v>15.84</v>
@@ -8057,7 +8058,7 @@
         </is>
       </c>
       <c r="D239" t="n">
-        <v>-24.55</v>
+        <v>-0.25</v>
       </c>
       <c r="E239" t="n">
         <v>0</v>
@@ -8089,10 +8090,10 @@
         </is>
       </c>
       <c r="D240" t="n">
-        <v>-24.55</v>
+        <v>-0.25</v>
       </c>
       <c r="E240" t="n">
-        <v>16.15</v>
+        <v>7.25</v>
       </c>
       <c r="F240" t="n">
         <v>15.84</v>
@@ -8121,10 +8122,10 @@
         </is>
       </c>
       <c r="D241" t="n">
-        <v>-15.8</v>
+        <v>-32.05</v>
       </c>
       <c r="E241" t="n">
-        <v>0</v>
+        <v>16.15</v>
       </c>
       <c r="F241" t="n">
         <v>15.84</v>
@@ -8153,7 +8154,7 @@
         </is>
       </c>
       <c r="D242" t="n">
-        <v>-15.8</v>
+        <v>-0.25</v>
       </c>
       <c r="E242" t="n">
         <v>16.15</v>
@@ -8185,10 +8186,10 @@
         </is>
       </c>
       <c r="D243" t="n">
-        <v>-5.8</v>
+        <v>-32.05</v>
       </c>
       <c r="E243" t="n">
-        <v>0</v>
+        <v>11.885</v>
       </c>
       <c r="F243" t="n">
         <v>15.84</v>
@@ -8217,10 +8218,10 @@
         </is>
       </c>
       <c r="D244" t="n">
-        <v>-5.8</v>
+        <v>-24.55</v>
       </c>
       <c r="E244" t="n">
-        <v>16.15</v>
+        <v>11.885</v>
       </c>
       <c r="F244" t="n">
         <v>15.84</v>
@@ -8241,7 +8242,7 @@
         <v>900090</v>
       </c>
       <c r="B245" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C245" t="inlineStr">
         <is>
@@ -8252,10 +8253,10 @@
         <v>-32.05</v>
       </c>
       <c r="E245" t="n">
-        <v>0</v>
+        <v>4.265</v>
       </c>
       <c r="F245" t="n">
-        <v>19.8</v>
+        <v>15.84</v>
       </c>
       <c r="G245" t="inlineStr">
         <is>
@@ -8273,7 +8274,7 @@
         <v>900091</v>
       </c>
       <c r="B246" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C246" t="inlineStr">
         <is>
@@ -8281,13 +8282,13 @@
         </is>
       </c>
       <c r="D246" t="n">
-        <v>-0.25</v>
+        <v>-24.55</v>
       </c>
       <c r="E246" t="n">
-        <v>0</v>
+        <v>4.265</v>
       </c>
       <c r="F246" t="n">
-        <v>19.8</v>
+        <v>15.84</v>
       </c>
       <c r="G246" t="inlineStr">
         <is>
@@ -8305,7 +8306,7 @@
         <v>900092</v>
       </c>
       <c r="B247" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C247" t="inlineStr">
         <is>
@@ -8313,13 +8314,13 @@
         </is>
       </c>
       <c r="D247" t="n">
-        <v>-0.25</v>
+        <v>-28.3</v>
       </c>
       <c r="E247" t="n">
-        <v>7.25</v>
+        <v>0</v>
       </c>
       <c r="F247" t="n">
-        <v>19.8</v>
+        <v>15.84</v>
       </c>
       <c r="G247" t="inlineStr">
         <is>
@@ -8337,7 +8338,7 @@
         <v>900093</v>
       </c>
       <c r="B248" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C248" t="inlineStr">
         <is>
@@ -8345,13 +8346,13 @@
         </is>
       </c>
       <c r="D248" t="n">
-        <v>-32.05</v>
+        <v>-28.3</v>
       </c>
       <c r="E248" t="n">
         <v>16.15</v>
       </c>
       <c r="F248" t="n">
-        <v>19.8</v>
+        <v>15.84</v>
       </c>
       <c r="G248" t="inlineStr">
         <is>
@@ -8369,7 +8370,7 @@
         <v>900094</v>
       </c>
       <c r="B249" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C249" t="inlineStr">
         <is>
@@ -8377,13 +8378,13 @@
         </is>
       </c>
       <c r="D249" t="n">
-        <v>-0.25</v>
+        <v>-24.55</v>
       </c>
       <c r="E249" t="n">
-        <v>16.15</v>
+        <v>0</v>
       </c>
       <c r="F249" t="n">
-        <v>19.8</v>
+        <v>15.84</v>
       </c>
       <c r="G249" t="inlineStr">
         <is>
@@ -8401,7 +8402,7 @@
         <v>900095</v>
       </c>
       <c r="B250" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C250" t="inlineStr">
         <is>
@@ -8409,13 +8410,13 @@
         </is>
       </c>
       <c r="D250" t="n">
-        <v>-32.05</v>
+        <v>-24.55</v>
       </c>
       <c r="E250" t="n">
-        <v>11.885</v>
+        <v>16.15</v>
       </c>
       <c r="F250" t="n">
-        <v>19.8</v>
+        <v>15.84</v>
       </c>
       <c r="G250" t="inlineStr">
         <is>
@@ -8433,7 +8434,7 @@
         <v>900096</v>
       </c>
       <c r="B251" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C251" t="inlineStr">
         <is>
@@ -8441,13 +8442,13 @@
         </is>
       </c>
       <c r="D251" t="n">
-        <v>-24.55</v>
+        <v>-15.8</v>
       </c>
       <c r="E251" t="n">
-        <v>11.885</v>
+        <v>0</v>
       </c>
       <c r="F251" t="n">
-        <v>19.8</v>
+        <v>15.84</v>
       </c>
       <c r="G251" t="inlineStr">
         <is>
@@ -8465,7 +8466,7 @@
         <v>900097</v>
       </c>
       <c r="B252" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C252" t="inlineStr">
         <is>
@@ -8473,13 +8474,13 @@
         </is>
       </c>
       <c r="D252" t="n">
-        <v>-32.05</v>
+        <v>-15.8</v>
       </c>
       <c r="E252" t="n">
-        <v>4.265</v>
+        <v>16.15</v>
       </c>
       <c r="F252" t="n">
-        <v>19.8</v>
+        <v>15.84</v>
       </c>
       <c r="G252" t="inlineStr">
         <is>
@@ -8497,7 +8498,7 @@
         <v>900098</v>
       </c>
       <c r="B253" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C253" t="inlineStr">
         <is>
@@ -8505,13 +8506,13 @@
         </is>
       </c>
       <c r="D253" t="n">
-        <v>-24.55</v>
+        <v>-5.8</v>
       </c>
       <c r="E253" t="n">
-        <v>4.265</v>
+        <v>0</v>
       </c>
       <c r="F253" t="n">
-        <v>19.8</v>
+        <v>15.84</v>
       </c>
       <c r="G253" t="inlineStr">
         <is>
@@ -8529,7 +8530,7 @@
         <v>900099</v>
       </c>
       <c r="B254" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C254" t="inlineStr">
         <is>
@@ -8537,13 +8538,13 @@
         </is>
       </c>
       <c r="D254" t="n">
-        <v>-28.3</v>
+        <v>-5.8</v>
       </c>
       <c r="E254" t="n">
-        <v>0</v>
+        <v>16.15</v>
       </c>
       <c r="F254" t="n">
-        <v>19.8</v>
+        <v>15.84</v>
       </c>
       <c r="G254" t="inlineStr">
         <is>
@@ -8569,10 +8570,10 @@
         </is>
       </c>
       <c r="D255" t="n">
-        <v>-28.3</v>
+        <v>-32.05</v>
       </c>
       <c r="E255" t="n">
-        <v>16.15</v>
+        <v>0</v>
       </c>
       <c r="F255" t="n">
         <v>19.8</v>
@@ -8601,7 +8602,7 @@
         </is>
       </c>
       <c r="D256" t="n">
-        <v>-24.55</v>
+        <v>-0.25</v>
       </c>
       <c r="E256" t="n">
         <v>0</v>
@@ -8633,10 +8634,10 @@
         </is>
       </c>
       <c r="D257" t="n">
-        <v>-24.55</v>
+        <v>-0.25</v>
       </c>
       <c r="E257" t="n">
-        <v>16.15</v>
+        <v>7.25</v>
       </c>
       <c r="F257" t="n">
         <v>19.8</v>
@@ -8665,10 +8666,10 @@
         </is>
       </c>
       <c r="D258" t="n">
-        <v>-15.8</v>
+        <v>-32.05</v>
       </c>
       <c r="E258" t="n">
-        <v>0</v>
+        <v>16.15</v>
       </c>
       <c r="F258" t="n">
         <v>19.8</v>
@@ -8697,7 +8698,7 @@
         </is>
       </c>
       <c r="D259" t="n">
-        <v>-15.8</v>
+        <v>-0.25</v>
       </c>
       <c r="E259" t="n">
         <v>16.15</v>
@@ -8729,10 +8730,10 @@
         </is>
       </c>
       <c r="D260" t="n">
-        <v>-5.8</v>
+        <v>-32.05</v>
       </c>
       <c r="E260" t="n">
-        <v>0</v>
+        <v>11.885</v>
       </c>
       <c r="F260" t="n">
         <v>19.8</v>
@@ -8761,10 +8762,10 @@
         </is>
       </c>
       <c r="D261" t="n">
-        <v>-5.8</v>
+        <v>-24.55</v>
       </c>
       <c r="E261" t="n">
-        <v>16.15</v>
+        <v>11.885</v>
       </c>
       <c r="F261" t="n">
         <v>19.8</v>
@@ -8785,7 +8786,7 @@
         <v>900107</v>
       </c>
       <c r="B262" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C262" t="inlineStr">
         <is>
@@ -8793,13 +8794,13 @@
         </is>
       </c>
       <c r="D262" t="n">
-        <v>10</v>
+        <v>-32.05</v>
       </c>
       <c r="E262" t="n">
-        <v>-4.12</v>
+        <v>4.265</v>
       </c>
       <c r="F262" t="n">
-        <v>11.88</v>
+        <v>19.8</v>
       </c>
       <c r="G262" t="inlineStr">
         <is>
@@ -8817,7 +8818,7 @@
         <v>900108</v>
       </c>
       <c r="B263" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C263" t="inlineStr">
         <is>
@@ -8825,13 +8826,13 @@
         </is>
       </c>
       <c r="D263" t="n">
-        <v>17.49</v>
+        <v>-24.55</v>
       </c>
       <c r="E263" t="n">
-        <v>-4.12</v>
+        <v>4.265</v>
       </c>
       <c r="F263" t="n">
-        <v>11.88</v>
+        <v>19.8</v>
       </c>
       <c r="G263" t="inlineStr">
         <is>
@@ -8849,7 +8850,7 @@
         <v>900109</v>
       </c>
       <c r="B264" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C264" t="inlineStr">
         <is>
@@ -8857,13 +8858,13 @@
         </is>
       </c>
       <c r="D264" t="n">
-        <v>15</v>
+        <v>-28.3</v>
       </c>
       <c r="E264" t="n">
         <v>0</v>
       </c>
       <c r="F264" t="n">
-        <v>11.88</v>
+        <v>19.8</v>
       </c>
       <c r="G264" t="inlineStr">
         <is>
@@ -8881,7 +8882,7 @@
         <v>900110</v>
       </c>
       <c r="B265" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C265" t="inlineStr">
         <is>
@@ -8889,13 +8890,13 @@
         </is>
       </c>
       <c r="D265" t="n">
-        <v>15</v>
+        <v>-28.3</v>
       </c>
       <c r="E265" t="n">
         <v>16.15</v>
       </c>
       <c r="F265" t="n">
-        <v>11.88</v>
+        <v>19.8</v>
       </c>
       <c r="G265" t="inlineStr">
         <is>
@@ -8913,7 +8914,7 @@
         <v>900111</v>
       </c>
       <c r="B266" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C266" t="inlineStr">
         <is>
@@ -8921,13 +8922,13 @@
         </is>
       </c>
       <c r="D266" t="n">
-        <v>25</v>
+        <v>-24.55</v>
       </c>
       <c r="E266" t="n">
-        <v>16.15</v>
+        <v>0</v>
       </c>
       <c r="F266" t="n">
-        <v>11.88</v>
+        <v>19.8</v>
       </c>
       <c r="G266" t="inlineStr">
         <is>
@@ -8945,7 +8946,7 @@
         <v>900112</v>
       </c>
       <c r="B267" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C267" t="inlineStr">
         <is>
@@ -8953,13 +8954,13 @@
         </is>
       </c>
       <c r="D267" t="n">
-        <v>17.49</v>
+        <v>-24.55</v>
       </c>
       <c r="E267" t="n">
-        <v>0</v>
+        <v>16.15</v>
       </c>
       <c r="F267" t="n">
-        <v>11.88</v>
+        <v>19.8</v>
       </c>
       <c r="G267" t="inlineStr">
         <is>
@@ -8977,7 +8978,7 @@
         <v>900113</v>
       </c>
       <c r="B268" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C268" t="inlineStr">
         <is>
@@ -8985,13 +8986,13 @@
         </is>
       </c>
       <c r="D268" t="n">
-        <v>17.49</v>
+        <v>-15.8</v>
       </c>
       <c r="E268" t="n">
-        <v>7.25</v>
+        <v>0</v>
       </c>
       <c r="F268" t="n">
-        <v>11.88</v>
+        <v>19.8</v>
       </c>
       <c r="G268" t="inlineStr">
         <is>
@@ -9009,7 +9010,7 @@
         <v>900114</v>
       </c>
       <c r="B269" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C269" t="inlineStr">
         <is>
@@ -9017,13 +9018,13 @@
         </is>
       </c>
       <c r="D269" t="n">
-        <v>35</v>
+        <v>-15.8</v>
       </c>
       <c r="E269" t="n">
-        <v>0</v>
+        <v>16.15</v>
       </c>
       <c r="F269" t="n">
-        <v>11.88</v>
+        <v>19.8</v>
       </c>
       <c r="G269" t="inlineStr">
         <is>
@@ -9041,7 +9042,7 @@
         <v>900115</v>
       </c>
       <c r="B270" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C270" t="inlineStr">
         <is>
@@ -9049,13 +9050,13 @@
         </is>
       </c>
       <c r="D270" t="n">
-        <v>35</v>
+        <v>-5.8</v>
       </c>
       <c r="E270" t="n">
-        <v>16.15</v>
+        <v>0</v>
       </c>
       <c r="F270" t="n">
-        <v>11.88</v>
+        <v>19.8</v>
       </c>
       <c r="G270" t="inlineStr">
         <is>
@@ -9073,7 +9074,7 @@
         <v>900116</v>
       </c>
       <c r="B271" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C271" t="inlineStr">
         <is>
@@ -9081,13 +9082,13 @@
         </is>
       </c>
       <c r="D271" t="n">
-        <v>15</v>
+        <v>-5.8</v>
       </c>
       <c r="E271" t="n">
-        <v>0</v>
+        <v>16.15</v>
       </c>
       <c r="F271" t="n">
-        <v>15.84</v>
+        <v>19.8</v>
       </c>
       <c r="G271" t="inlineStr">
         <is>
@@ -9105,7 +9106,7 @@
         <v>900117</v>
       </c>
       <c r="B272" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C272" t="inlineStr">
         <is>
@@ -9113,13 +9114,13 @@
         </is>
       </c>
       <c r="D272" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="E272" t="n">
-        <v>16.15</v>
+        <v>-4.12</v>
       </c>
       <c r="F272" t="n">
-        <v>15.84</v>
+        <v>11.88</v>
       </c>
       <c r="G272" t="inlineStr">
         <is>
@@ -9137,7 +9138,7 @@
         <v>900118</v>
       </c>
       <c r="B273" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C273" t="inlineStr">
         <is>
@@ -9145,13 +9146,13 @@
         </is>
       </c>
       <c r="D273" t="n">
-        <v>25</v>
+        <v>17.49</v>
       </c>
       <c r="E273" t="n">
-        <v>0</v>
+        <v>-4.12</v>
       </c>
       <c r="F273" t="n">
-        <v>15.84</v>
+        <v>11.88</v>
       </c>
       <c r="G273" t="inlineStr">
         <is>
@@ -9169,7 +9170,7 @@
         <v>900119</v>
       </c>
       <c r="B274" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C274" t="inlineStr">
         <is>
@@ -9177,13 +9178,13 @@
         </is>
       </c>
       <c r="D274" t="n">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="E274" t="n">
-        <v>16.15</v>
+        <v>0</v>
       </c>
       <c r="F274" t="n">
-        <v>15.84</v>
+        <v>11.88</v>
       </c>
       <c r="G274" t="inlineStr">
         <is>
@@ -9201,7 +9202,7 @@
         <v>900120</v>
       </c>
       <c r="B275" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C275" t="inlineStr">
         <is>
@@ -9209,13 +9210,13 @@
         </is>
       </c>
       <c r="D275" t="n">
-        <v>17.49</v>
+        <v>15</v>
       </c>
       <c r="E275" t="n">
-        <v>0</v>
+        <v>16.15</v>
       </c>
       <c r="F275" t="n">
-        <v>15.84</v>
+        <v>11.88</v>
       </c>
       <c r="G275" t="inlineStr">
         <is>
@@ -9233,7 +9234,7 @@
         <v>900121</v>
       </c>
       <c r="B276" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C276" t="inlineStr">
         <is>
@@ -9241,13 +9242,13 @@
         </is>
       </c>
       <c r="D276" t="n">
-        <v>17.49</v>
+        <v>25</v>
       </c>
       <c r="E276" t="n">
-        <v>7.25</v>
+        <v>16.15</v>
       </c>
       <c r="F276" t="n">
-        <v>15.84</v>
+        <v>11.88</v>
       </c>
       <c r="G276" t="inlineStr">
         <is>
@@ -9265,7 +9266,7 @@
         <v>900122</v>
       </c>
       <c r="B277" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C277" t="inlineStr">
         <is>
@@ -9273,13 +9274,13 @@
         </is>
       </c>
       <c r="D277" t="n">
-        <v>35</v>
+        <v>17.49</v>
       </c>
       <c r="E277" t="n">
         <v>0</v>
       </c>
       <c r="F277" t="n">
-        <v>15.84</v>
+        <v>11.88</v>
       </c>
       <c r="G277" t="inlineStr">
         <is>
@@ -9297,28 +9298,348 @@
         <v>900123</v>
       </c>
       <c r="B278" t="n">
+        <v>3</v>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>BEAM_MANUAL</t>
+        </is>
+      </c>
+      <c r="D278" t="n">
+        <v>17.49</v>
+      </c>
+      <c r="E278" t="n">
+        <v>7.25</v>
+      </c>
+      <c r="F278" t="n">
+        <v>11.88</v>
+      </c>
+      <c r="G278" t="inlineStr">
+        <is>
+          <t>Libre</t>
+        </is>
+      </c>
+      <c r="H278" t="inlineStr">
+        <is>
+          <t>MANUAL_BEAM_NODE</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="n">
+        <v>900124</v>
+      </c>
+      <c r="B279" t="n">
+        <v>3</v>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>BEAM_MANUAL</t>
+        </is>
+      </c>
+      <c r="D279" t="n">
+        <v>35</v>
+      </c>
+      <c r="E279" t="n">
+        <v>0</v>
+      </c>
+      <c r="F279" t="n">
+        <v>11.88</v>
+      </c>
+      <c r="G279" t="inlineStr">
+        <is>
+          <t>Libre</t>
+        </is>
+      </c>
+      <c r="H279" t="inlineStr">
+        <is>
+          <t>MANUAL_BEAM_NODE</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="n">
+        <v>900125</v>
+      </c>
+      <c r="B280" t="n">
+        <v>3</v>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>BEAM_MANUAL</t>
+        </is>
+      </c>
+      <c r="D280" t="n">
+        <v>35</v>
+      </c>
+      <c r="E280" t="n">
+        <v>16.15</v>
+      </c>
+      <c r="F280" t="n">
+        <v>11.88</v>
+      </c>
+      <c r="G280" t="inlineStr">
+        <is>
+          <t>Libre</t>
+        </is>
+      </c>
+      <c r="H280" t="inlineStr">
+        <is>
+          <t>MANUAL_BEAM_NODE</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="n">
+        <v>900126</v>
+      </c>
+      <c r="B281" t="n">
         <v>4</v>
       </c>
-      <c r="C278" t="inlineStr">
+      <c r="C281" t="inlineStr">
         <is>
           <t>BEAM_MANUAL</t>
         </is>
       </c>
-      <c r="D278" t="n">
+      <c r="D281" t="n">
+        <v>15</v>
+      </c>
+      <c r="E281" t="n">
+        <v>0</v>
+      </c>
+      <c r="F281" t="n">
+        <v>15.84</v>
+      </c>
+      <c r="G281" t="inlineStr">
+        <is>
+          <t>Libre</t>
+        </is>
+      </c>
+      <c r="H281" t="inlineStr">
+        <is>
+          <t>MANUAL_BEAM_NODE</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="n">
+        <v>900127</v>
+      </c>
+      <c r="B282" t="n">
+        <v>4</v>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>BEAM_MANUAL</t>
+        </is>
+      </c>
+      <c r="D282" t="n">
+        <v>15</v>
+      </c>
+      <c r="E282" t="n">
+        <v>16.15</v>
+      </c>
+      <c r="F282" t="n">
+        <v>15.84</v>
+      </c>
+      <c r="G282" t="inlineStr">
+        <is>
+          <t>Libre</t>
+        </is>
+      </c>
+      <c r="H282" t="inlineStr">
+        <is>
+          <t>MANUAL_BEAM_NODE</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="n">
+        <v>900128</v>
+      </c>
+      <c r="B283" t="n">
+        <v>4</v>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>BEAM_MANUAL</t>
+        </is>
+      </c>
+      <c r="D283" t="n">
+        <v>25</v>
+      </c>
+      <c r="E283" t="n">
+        <v>0</v>
+      </c>
+      <c r="F283" t="n">
+        <v>15.84</v>
+      </c>
+      <c r="G283" t="inlineStr">
+        <is>
+          <t>Libre</t>
+        </is>
+      </c>
+      <c r="H283" t="inlineStr">
+        <is>
+          <t>MANUAL_BEAM_NODE</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="n">
+        <v>900129</v>
+      </c>
+      <c r="B284" t="n">
+        <v>4</v>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>BEAM_MANUAL</t>
+        </is>
+      </c>
+      <c r="D284" t="n">
+        <v>25</v>
+      </c>
+      <c r="E284" t="n">
+        <v>16.15</v>
+      </c>
+      <c r="F284" t="n">
+        <v>15.84</v>
+      </c>
+      <c r="G284" t="inlineStr">
+        <is>
+          <t>Libre</t>
+        </is>
+      </c>
+      <c r="H284" t="inlineStr">
+        <is>
+          <t>MANUAL_BEAM_NODE</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="n">
+        <v>900130</v>
+      </c>
+      <c r="B285" t="n">
+        <v>4</v>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>BEAM_MANUAL</t>
+        </is>
+      </c>
+      <c r="D285" t="n">
+        <v>17.49</v>
+      </c>
+      <c r="E285" t="n">
+        <v>0</v>
+      </c>
+      <c r="F285" t="n">
+        <v>15.84</v>
+      </c>
+      <c r="G285" t="inlineStr">
+        <is>
+          <t>Libre</t>
+        </is>
+      </c>
+      <c r="H285" t="inlineStr">
+        <is>
+          <t>MANUAL_BEAM_NODE</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="n">
+        <v>900131</v>
+      </c>
+      <c r="B286" t="n">
+        <v>4</v>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>BEAM_MANUAL</t>
+        </is>
+      </c>
+      <c r="D286" t="n">
+        <v>17.49</v>
+      </c>
+      <c r="E286" t="n">
+        <v>7.25</v>
+      </c>
+      <c r="F286" t="n">
+        <v>15.84</v>
+      </c>
+      <c r="G286" t="inlineStr">
+        <is>
+          <t>Libre</t>
+        </is>
+      </c>
+      <c r="H286" t="inlineStr">
+        <is>
+          <t>MANUAL_BEAM_NODE</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="n">
+        <v>900132</v>
+      </c>
+      <c r="B287" t="n">
+        <v>4</v>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>BEAM_MANUAL</t>
+        </is>
+      </c>
+      <c r="D287" t="n">
         <v>35</v>
       </c>
-      <c r="E278" t="n">
+      <c r="E287" t="n">
+        <v>0</v>
+      </c>
+      <c r="F287" t="n">
+        <v>15.84</v>
+      </c>
+      <c r="G287" t="inlineStr">
+        <is>
+          <t>Libre</t>
+        </is>
+      </c>
+      <c r="H287" t="inlineStr">
+        <is>
+          <t>MANUAL_BEAM_NODE</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="n">
+        <v>900133</v>
+      </c>
+      <c r="B288" t="n">
+        <v>4</v>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>BEAM_MANUAL</t>
+        </is>
+      </c>
+      <c r="D288" t="n">
+        <v>35</v>
+      </c>
+      <c r="E288" t="n">
         <v>16.15</v>
       </c>
-      <c r="F278" t="n">
+      <c r="F288" t="n">
         <v>15.84</v>
       </c>
-      <c r="G278" t="inlineStr">
-        <is>
-          <t>Libre</t>
-        </is>
-      </c>
-      <c r="H278" t="inlineStr">
+      <c r="G288" t="inlineStr">
+        <is>
+          <t>Libre</t>
+        </is>
+      </c>
+      <c r="H288" t="inlineStr">
         <is>
           <t>MANUAL_BEAM_NODE</t>
         </is>
@@ -9335,7 +9656,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E254"/>
+  <dimension ref="A1:E271"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13071,10 +13392,10 @@
         </is>
       </c>
       <c r="C178" t="n">
-        <v>900039</v>
+        <v>502001</v>
       </c>
       <c r="D178" t="n">
-        <v>900040</v>
+        <v>502501</v>
       </c>
       <c r="E178" t="inlineStr">
         <is>
@@ -13092,10 +13413,10 @@
         </is>
       </c>
       <c r="C179" t="n">
-        <v>702004</v>
+        <v>501001</v>
       </c>
       <c r="D179" t="n">
-        <v>900041</v>
+        <v>501501</v>
       </c>
       <c r="E179" t="inlineStr">
         <is>
@@ -13113,10 +13434,10 @@
         </is>
       </c>
       <c r="C180" t="n">
-        <v>900042</v>
+        <v>500001</v>
       </c>
       <c r="D180" t="n">
-        <v>900043</v>
+        <v>500501</v>
       </c>
       <c r="E180" t="inlineStr">
         <is>
@@ -13130,14 +13451,14 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>BEAM_X</t>
+          <t>BEAM_Y</t>
         </is>
       </c>
       <c r="C181" t="n">
-        <v>900044</v>
+        <v>500001</v>
       </c>
       <c r="D181" t="n">
-        <v>900045</v>
+        <v>502001</v>
       </c>
       <c r="E181" t="inlineStr">
         <is>
@@ -13151,14 +13472,14 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>BEAM_X</t>
+          <t>BEAM_Y</t>
         </is>
       </c>
       <c r="C182" t="n">
-        <v>900046</v>
+        <v>500101</v>
       </c>
       <c r="D182" t="n">
-        <v>900047</v>
+        <v>502101</v>
       </c>
       <c r="E182" t="inlineStr">
         <is>
@@ -13176,10 +13497,10 @@
         </is>
       </c>
       <c r="C183" t="n">
-        <v>900039</v>
+        <v>500201</v>
       </c>
       <c r="D183" t="n">
-        <v>900042</v>
+        <v>502201</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
@@ -13197,10 +13518,10 @@
         </is>
       </c>
       <c r="C184" t="n">
-        <v>900048</v>
+        <v>500301</v>
       </c>
       <c r="D184" t="n">
-        <v>900049</v>
+        <v>502301</v>
       </c>
       <c r="E184" t="inlineStr">
         <is>
@@ -13218,10 +13539,10 @@
         </is>
       </c>
       <c r="C185" t="n">
-        <v>702007</v>
+        <v>500401</v>
       </c>
       <c r="D185" t="n">
-        <v>702001</v>
+        <v>502401</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
@@ -13239,10 +13560,10 @@
         </is>
       </c>
       <c r="C186" t="n">
-        <v>702008</v>
+        <v>500451</v>
       </c>
       <c r="D186" t="n">
-        <v>702002</v>
+        <v>502451</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
@@ -13260,10 +13581,10 @@
         </is>
       </c>
       <c r="C187" t="n">
-        <v>900050</v>
+        <v>500501</v>
       </c>
       <c r="D187" t="n">
-        <v>900051</v>
+        <v>502501</v>
       </c>
       <c r="E187" t="inlineStr">
         <is>
@@ -13281,10 +13602,10 @@
         </is>
       </c>
       <c r="C188" t="n">
-        <v>900052</v>
+        <v>900039</v>
       </c>
       <c r="D188" t="n">
-        <v>900053</v>
+        <v>900040</v>
       </c>
       <c r="E188" t="inlineStr">
         <is>
@@ -13302,10 +13623,10 @@
         </is>
       </c>
       <c r="C189" t="n">
-        <v>900054</v>
+        <v>900041</v>
       </c>
       <c r="D189" t="n">
-        <v>900055</v>
+        <v>900042</v>
       </c>
       <c r="E189" t="inlineStr">
         <is>
@@ -13319,14 +13640,14 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>BEAM_X</t>
+          <t>BEAM_Y</t>
         </is>
       </c>
       <c r="C190" t="n">
-        <v>900056</v>
+        <v>900043</v>
       </c>
       <c r="D190" t="n">
-        <v>900057</v>
+        <v>900044</v>
       </c>
       <c r="E190" t="inlineStr">
         <is>
@@ -13340,14 +13661,14 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>BEAM_X</t>
+          <t>BEAM_Y</t>
         </is>
       </c>
       <c r="C191" t="n">
-        <v>703004</v>
+        <v>900045</v>
       </c>
       <c r="D191" t="n">
-        <v>900058</v>
+        <v>900046</v>
       </c>
       <c r="E191" t="inlineStr">
         <is>
@@ -13361,14 +13682,14 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>BEAM_X</t>
+          <t>BEAM_Y</t>
         </is>
       </c>
       <c r="C192" t="n">
-        <v>900059</v>
+        <v>900047</v>
       </c>
       <c r="D192" t="n">
-        <v>900060</v>
+        <v>500201</v>
       </c>
       <c r="E192" t="inlineStr">
         <is>
@@ -13382,14 +13703,14 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>BEAM_X</t>
+          <t>BEAM_Y</t>
         </is>
       </c>
       <c r="C193" t="n">
-        <v>900061</v>
+        <v>900048</v>
       </c>
       <c r="D193" t="n">
-        <v>900062</v>
+        <v>500301</v>
       </c>
       <c r="E193" t="inlineStr">
         <is>
@@ -13407,10 +13728,10 @@
         </is>
       </c>
       <c r="C194" t="n">
-        <v>900063</v>
+        <v>900047</v>
       </c>
       <c r="D194" t="n">
-        <v>900064</v>
+        <v>900048</v>
       </c>
       <c r="E194" t="inlineStr">
         <is>
@@ -13424,14 +13745,14 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>BEAM_Y</t>
+          <t>BEAM_X</t>
         </is>
       </c>
       <c r="C195" t="n">
-        <v>900056</v>
+        <v>900049</v>
       </c>
       <c r="D195" t="n">
-        <v>900059</v>
+        <v>900050</v>
       </c>
       <c r="E195" t="inlineStr">
         <is>
@@ -13445,14 +13766,14 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>BEAM_Y</t>
+          <t>BEAM_X</t>
         </is>
       </c>
       <c r="C196" t="n">
-        <v>900065</v>
+        <v>702004</v>
       </c>
       <c r="D196" t="n">
-        <v>900066</v>
+        <v>900051</v>
       </c>
       <c r="E196" t="inlineStr">
         <is>
@@ -13466,14 +13787,14 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>BEAM_Y</t>
+          <t>BEAM_X</t>
         </is>
       </c>
       <c r="C197" t="n">
-        <v>703007</v>
+        <v>900052</v>
       </c>
       <c r="D197" t="n">
-        <v>703001</v>
+        <v>900053</v>
       </c>
       <c r="E197" t="inlineStr">
         <is>
@@ -13487,14 +13808,14 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>BEAM_Y</t>
+          <t>BEAM_X</t>
         </is>
       </c>
       <c r="C198" t="n">
-        <v>703008</v>
+        <v>900054</v>
       </c>
       <c r="D198" t="n">
-        <v>703002</v>
+        <v>900055</v>
       </c>
       <c r="E198" t="inlineStr">
         <is>
@@ -13508,14 +13829,14 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>BEAM_Y</t>
+          <t>BEAM_X</t>
         </is>
       </c>
       <c r="C199" t="n">
-        <v>900067</v>
+        <v>900056</v>
       </c>
       <c r="D199" t="n">
-        <v>900068</v>
+        <v>900057</v>
       </c>
       <c r="E199" t="inlineStr">
         <is>
@@ -13533,10 +13854,10 @@
         </is>
       </c>
       <c r="C200" t="n">
-        <v>900069</v>
+        <v>900049</v>
       </c>
       <c r="D200" t="n">
-        <v>900070</v>
+        <v>900052</v>
       </c>
       <c r="E200" t="inlineStr">
         <is>
@@ -13554,10 +13875,10 @@
         </is>
       </c>
       <c r="C201" t="n">
-        <v>900071</v>
+        <v>900058</v>
       </c>
       <c r="D201" t="n">
-        <v>900072</v>
+        <v>900059</v>
       </c>
       <c r="E201" t="inlineStr">
         <is>
@@ -13571,14 +13892,14 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>BEAM_X</t>
+          <t>BEAM_Y</t>
         </is>
       </c>
       <c r="C202" t="n">
-        <v>900073</v>
+        <v>702007</v>
       </c>
       <c r="D202" t="n">
-        <v>900074</v>
+        <v>702001</v>
       </c>
       <c r="E202" t="inlineStr">
         <is>
@@ -13592,14 +13913,14 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>BEAM_X</t>
+          <t>BEAM_Y</t>
         </is>
       </c>
       <c r="C203" t="n">
-        <v>704004</v>
+        <v>702008</v>
       </c>
       <c r="D203" t="n">
-        <v>900075</v>
+        <v>702002</v>
       </c>
       <c r="E203" t="inlineStr">
         <is>
@@ -13613,14 +13934,14 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>BEAM_X</t>
+          <t>BEAM_Y</t>
         </is>
       </c>
       <c r="C204" t="n">
-        <v>900076</v>
+        <v>900060</v>
       </c>
       <c r="D204" t="n">
-        <v>900077</v>
+        <v>900061</v>
       </c>
       <c r="E204" t="inlineStr">
         <is>
@@ -13634,14 +13955,14 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>BEAM_X</t>
+          <t>BEAM_Y</t>
         </is>
       </c>
       <c r="C205" t="n">
-        <v>900078</v>
+        <v>900062</v>
       </c>
       <c r="D205" t="n">
-        <v>900079</v>
+        <v>900063</v>
       </c>
       <c r="E205" t="inlineStr">
         <is>
@@ -13655,14 +13976,14 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>BEAM_X</t>
+          <t>BEAM_Y</t>
         </is>
       </c>
       <c r="C206" t="n">
-        <v>900080</v>
+        <v>900064</v>
       </c>
       <c r="D206" t="n">
-        <v>900081</v>
+        <v>900065</v>
       </c>
       <c r="E206" t="inlineStr">
         <is>
@@ -13676,14 +13997,14 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>BEAM_Y</t>
+          <t>BEAM_X</t>
         </is>
       </c>
       <c r="C207" t="n">
-        <v>900073</v>
+        <v>900066</v>
       </c>
       <c r="D207" t="n">
-        <v>900076</v>
+        <v>900067</v>
       </c>
       <c r="E207" t="inlineStr">
         <is>
@@ -13697,14 +14018,14 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>BEAM_Y</t>
+          <t>BEAM_X</t>
         </is>
       </c>
       <c r="C208" t="n">
-        <v>900082</v>
+        <v>703004</v>
       </c>
       <c r="D208" t="n">
-        <v>900083</v>
+        <v>900068</v>
       </c>
       <c r="E208" t="inlineStr">
         <is>
@@ -13718,14 +14039,14 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>BEAM_Y</t>
+          <t>BEAM_X</t>
         </is>
       </c>
       <c r="C209" t="n">
-        <v>704007</v>
+        <v>900069</v>
       </c>
       <c r="D209" t="n">
-        <v>704001</v>
+        <v>900070</v>
       </c>
       <c r="E209" t="inlineStr">
         <is>
@@ -13739,14 +14060,14 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>BEAM_Y</t>
+          <t>BEAM_X</t>
         </is>
       </c>
       <c r="C210" t="n">
-        <v>704008</v>
+        <v>900071</v>
       </c>
       <c r="D210" t="n">
-        <v>704002</v>
+        <v>900072</v>
       </c>
       <c r="E210" t="inlineStr">
         <is>
@@ -13760,14 +14081,14 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>BEAM_Y</t>
+          <t>BEAM_X</t>
         </is>
       </c>
       <c r="C211" t="n">
-        <v>900084</v>
+        <v>900073</v>
       </c>
       <c r="D211" t="n">
-        <v>900085</v>
+        <v>900074</v>
       </c>
       <c r="E211" t="inlineStr">
         <is>
@@ -13785,10 +14106,10 @@
         </is>
       </c>
       <c r="C212" t="n">
-        <v>900086</v>
+        <v>900066</v>
       </c>
       <c r="D212" t="n">
-        <v>900087</v>
+        <v>900069</v>
       </c>
       <c r="E212" t="inlineStr">
         <is>
@@ -13806,10 +14127,10 @@
         </is>
       </c>
       <c r="C213" t="n">
-        <v>900088</v>
+        <v>900075</v>
       </c>
       <c r="D213" t="n">
-        <v>900089</v>
+        <v>900076</v>
       </c>
       <c r="E213" t="inlineStr">
         <is>
@@ -13823,14 +14144,14 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>BEAM_X</t>
+          <t>BEAM_Y</t>
         </is>
       </c>
       <c r="C214" t="n">
-        <v>900090</v>
+        <v>703007</v>
       </c>
       <c r="D214" t="n">
-        <v>900091</v>
+        <v>703001</v>
       </c>
       <c r="E214" t="inlineStr">
         <is>
@@ -13844,14 +14165,14 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>BEAM_X</t>
+          <t>BEAM_Y</t>
         </is>
       </c>
       <c r="C215" t="n">
-        <v>705004</v>
+        <v>703008</v>
       </c>
       <c r="D215" t="n">
-        <v>900092</v>
+        <v>703002</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
@@ -13865,14 +14186,14 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>BEAM_X</t>
+          <t>BEAM_Y</t>
         </is>
       </c>
       <c r="C216" t="n">
-        <v>900093</v>
+        <v>900077</v>
       </c>
       <c r="D216" t="n">
-        <v>900094</v>
+        <v>900078</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
@@ -13886,14 +14207,14 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>BEAM_X</t>
+          <t>BEAM_Y</t>
         </is>
       </c>
       <c r="C217" t="n">
-        <v>900095</v>
+        <v>900079</v>
       </c>
       <c r="D217" t="n">
-        <v>900096</v>
+        <v>900080</v>
       </c>
       <c r="E217" t="inlineStr">
         <is>
@@ -13907,14 +14228,14 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>BEAM_X</t>
+          <t>BEAM_Y</t>
         </is>
       </c>
       <c r="C218" t="n">
-        <v>900097</v>
+        <v>900081</v>
       </c>
       <c r="D218" t="n">
-        <v>900098</v>
+        <v>900082</v>
       </c>
       <c r="E218" t="inlineStr">
         <is>
@@ -13928,14 +14249,14 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>BEAM_Y</t>
+          <t>BEAM_X</t>
         </is>
       </c>
       <c r="C219" t="n">
-        <v>900090</v>
+        <v>900083</v>
       </c>
       <c r="D219" t="n">
-        <v>900093</v>
+        <v>900084</v>
       </c>
       <c r="E219" t="inlineStr">
         <is>
@@ -13949,14 +14270,14 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>BEAM_Y</t>
+          <t>BEAM_X</t>
         </is>
       </c>
       <c r="C220" t="n">
-        <v>900099</v>
+        <v>704004</v>
       </c>
       <c r="D220" t="n">
-        <v>900100</v>
+        <v>900085</v>
       </c>
       <c r="E220" t="inlineStr">
         <is>
@@ -13970,14 +14291,14 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>BEAM_Y</t>
+          <t>BEAM_X</t>
         </is>
       </c>
       <c r="C221" t="n">
-        <v>705007</v>
+        <v>900086</v>
       </c>
       <c r="D221" t="n">
-        <v>705001</v>
+        <v>900087</v>
       </c>
       <c r="E221" t="inlineStr">
         <is>
@@ -13991,14 +14312,14 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>BEAM_Y</t>
+          <t>BEAM_X</t>
         </is>
       </c>
       <c r="C222" t="n">
-        <v>705008</v>
+        <v>900088</v>
       </c>
       <c r="D222" t="n">
-        <v>705002</v>
+        <v>900089</v>
       </c>
       <c r="E222" t="inlineStr">
         <is>
@@ -14012,14 +14333,14 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>BEAM_Y</t>
+          <t>BEAM_X</t>
         </is>
       </c>
       <c r="C223" t="n">
-        <v>900101</v>
+        <v>900090</v>
       </c>
       <c r="D223" t="n">
-        <v>900102</v>
+        <v>900091</v>
       </c>
       <c r="E223" t="inlineStr">
         <is>
@@ -14037,10 +14358,10 @@
         </is>
       </c>
       <c r="C224" t="n">
-        <v>900103</v>
+        <v>900083</v>
       </c>
       <c r="D224" t="n">
-        <v>900104</v>
+        <v>900086</v>
       </c>
       <c r="E224" t="inlineStr">
         <is>
@@ -14058,10 +14379,10 @@
         </is>
       </c>
       <c r="C225" t="n">
-        <v>900105</v>
+        <v>900092</v>
       </c>
       <c r="D225" t="n">
-        <v>900106</v>
+        <v>900093</v>
       </c>
       <c r="E225" t="inlineStr">
         <is>
@@ -14075,14 +14396,14 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>BEAM_X</t>
+          <t>BEAM_Y</t>
         </is>
       </c>
       <c r="C226" t="n">
-        <v>300001</v>
+        <v>704007</v>
       </c>
       <c r="D226" t="n">
-        <v>300451</v>
+        <v>704001</v>
       </c>
       <c r="E226" t="inlineStr">
         <is>
@@ -14096,14 +14417,14 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>BEAM_X</t>
+          <t>BEAM_Y</t>
         </is>
       </c>
       <c r="C227" t="n">
-        <v>301001</v>
+        <v>704008</v>
       </c>
       <c r="D227" t="n">
-        <v>301451</v>
+        <v>704002</v>
       </c>
       <c r="E227" t="inlineStr">
         <is>
@@ -14117,14 +14438,14 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>BEAM_X</t>
+          <t>BEAM_Y</t>
         </is>
       </c>
       <c r="C228" t="n">
-        <v>302001</v>
+        <v>900094</v>
       </c>
       <c r="D228" t="n">
-        <v>302451</v>
+        <v>900095</v>
       </c>
       <c r="E228" t="inlineStr">
         <is>
@@ -14138,14 +14459,14 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>BEAM_X</t>
+          <t>BEAM_Y</t>
         </is>
       </c>
       <c r="C229" t="n">
-        <v>900107</v>
+        <v>900096</v>
       </c>
       <c r="D229" t="n">
-        <v>900108</v>
+        <v>900097</v>
       </c>
       <c r="E229" t="inlineStr">
         <is>
@@ -14163,10 +14484,10 @@
         </is>
       </c>
       <c r="C230" t="n">
-        <v>300001</v>
+        <v>900098</v>
       </c>
       <c r="D230" t="n">
-        <v>302001</v>
+        <v>900099</v>
       </c>
       <c r="E230" t="inlineStr">
         <is>
@@ -14180,14 +14501,14 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>BEAM_Y</t>
+          <t>BEAM_X</t>
         </is>
       </c>
       <c r="C231" t="n">
-        <v>300101</v>
+        <v>900100</v>
       </c>
       <c r="D231" t="n">
-        <v>302101</v>
+        <v>900101</v>
       </c>
       <c r="E231" t="inlineStr">
         <is>
@@ -14201,14 +14522,14 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>BEAM_Y</t>
+          <t>BEAM_X</t>
         </is>
       </c>
       <c r="C232" t="n">
-        <v>300201</v>
+        <v>705004</v>
       </c>
       <c r="D232" t="n">
-        <v>302201</v>
+        <v>900102</v>
       </c>
       <c r="E232" t="inlineStr">
         <is>
@@ -14222,14 +14543,14 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>BEAM_Y</t>
+          <t>BEAM_X</t>
         </is>
       </c>
       <c r="C233" t="n">
-        <v>300301</v>
+        <v>900103</v>
       </c>
       <c r="D233" t="n">
-        <v>302301</v>
+        <v>900104</v>
       </c>
       <c r="E233" t="inlineStr">
         <is>
@@ -14243,14 +14564,14 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>BEAM_Y</t>
+          <t>BEAM_X</t>
         </is>
       </c>
       <c r="C234" t="n">
-        <v>300401</v>
+        <v>900105</v>
       </c>
       <c r="D234" t="n">
-        <v>302401</v>
+        <v>900106</v>
       </c>
       <c r="E234" t="inlineStr">
         <is>
@@ -14264,14 +14585,14 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>BEAM_Y</t>
+          <t>BEAM_X</t>
         </is>
       </c>
       <c r="C235" t="n">
-        <v>300451</v>
+        <v>900107</v>
       </c>
       <c r="D235" t="n">
-        <v>302451</v>
+        <v>900108</v>
       </c>
       <c r="E235" t="inlineStr">
         <is>
@@ -14289,10 +14610,10 @@
         </is>
       </c>
       <c r="C236" t="n">
-        <v>900107</v>
+        <v>900100</v>
       </c>
       <c r="D236" t="n">
-        <v>300101</v>
+        <v>900103</v>
       </c>
       <c r="E236" t="inlineStr">
         <is>
@@ -14331,10 +14652,10 @@
         </is>
       </c>
       <c r="C238" t="n">
-        <v>900028</v>
+        <v>705007</v>
       </c>
       <c r="D238" t="n">
-        <v>900111</v>
+        <v>705001</v>
       </c>
       <c r="E238" t="inlineStr">
         <is>
@@ -14352,10 +14673,10 @@
         </is>
       </c>
       <c r="C239" t="n">
-        <v>900112</v>
+        <v>705008</v>
       </c>
       <c r="D239" t="n">
-        <v>900113</v>
+        <v>705002</v>
       </c>
       <c r="E239" t="inlineStr">
         <is>
@@ -14373,7 +14694,7 @@
         </is>
       </c>
       <c r="C240" t="n">
-        <v>900108</v>
+        <v>900111</v>
       </c>
       <c r="D240" t="n">
         <v>900112</v>
@@ -14394,10 +14715,10 @@
         </is>
       </c>
       <c r="C241" t="n">
+        <v>900113</v>
+      </c>
+      <c r="D241" t="n">
         <v>900114</v>
-      </c>
-      <c r="D241" t="n">
-        <v>900115</v>
       </c>
       <c r="E241" t="inlineStr">
         <is>
@@ -14411,14 +14732,14 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>BEAM_X</t>
+          <t>BEAM_Y</t>
         </is>
       </c>
       <c r="C242" t="n">
-        <v>400001</v>
+        <v>900115</v>
       </c>
       <c r="D242" t="n">
-        <v>400451</v>
+        <v>900116</v>
       </c>
       <c r="E242" t="inlineStr">
         <is>
@@ -14436,10 +14757,10 @@
         </is>
       </c>
       <c r="C243" t="n">
-        <v>401001</v>
+        <v>300001</v>
       </c>
       <c r="D243" t="n">
-        <v>401451</v>
+        <v>300451</v>
       </c>
       <c r="E243" t="inlineStr">
         <is>
@@ -14457,10 +14778,10 @@
         </is>
       </c>
       <c r="C244" t="n">
-        <v>402001</v>
+        <v>301001</v>
       </c>
       <c r="D244" t="n">
-        <v>402451</v>
+        <v>301451</v>
       </c>
       <c r="E244" t="inlineStr">
         <is>
@@ -14474,14 +14795,14 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>BEAM_Y</t>
+          <t>BEAM_X</t>
         </is>
       </c>
       <c r="C245" t="n">
-        <v>400001</v>
+        <v>302001</v>
       </c>
       <c r="D245" t="n">
-        <v>402001</v>
+        <v>302451</v>
       </c>
       <c r="E245" t="inlineStr">
         <is>
@@ -14495,14 +14816,14 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>BEAM_Y</t>
+          <t>BEAM_X</t>
         </is>
       </c>
       <c r="C246" t="n">
-        <v>400101</v>
+        <v>900117</v>
       </c>
       <c r="D246" t="n">
-        <v>402101</v>
+        <v>900118</v>
       </c>
       <c r="E246" t="inlineStr">
         <is>
@@ -14520,10 +14841,10 @@
         </is>
       </c>
       <c r="C247" t="n">
-        <v>400201</v>
+        <v>300001</v>
       </c>
       <c r="D247" t="n">
-        <v>402201</v>
+        <v>302001</v>
       </c>
       <c r="E247" t="inlineStr">
         <is>
@@ -14541,10 +14862,10 @@
         </is>
       </c>
       <c r="C248" t="n">
-        <v>400301</v>
+        <v>300101</v>
       </c>
       <c r="D248" t="n">
-        <v>402301</v>
+        <v>302101</v>
       </c>
       <c r="E248" t="inlineStr">
         <is>
@@ -14562,10 +14883,10 @@
         </is>
       </c>
       <c r="C249" t="n">
-        <v>400401</v>
+        <v>300201</v>
       </c>
       <c r="D249" t="n">
-        <v>402401</v>
+        <v>302201</v>
       </c>
       <c r="E249" t="inlineStr">
         <is>
@@ -14583,10 +14904,10 @@
         </is>
       </c>
       <c r="C250" t="n">
-        <v>400451</v>
+        <v>300301</v>
       </c>
       <c r="D250" t="n">
-        <v>402451</v>
+        <v>302301</v>
       </c>
       <c r="E250" t="inlineStr">
         <is>
@@ -14604,10 +14925,10 @@
         </is>
       </c>
       <c r="C251" t="n">
-        <v>900116</v>
+        <v>300401</v>
       </c>
       <c r="D251" t="n">
-        <v>900117</v>
+        <v>302401</v>
       </c>
       <c r="E251" t="inlineStr">
         <is>
@@ -14625,10 +14946,10 @@
         </is>
       </c>
       <c r="C252" t="n">
-        <v>900118</v>
+        <v>300451</v>
       </c>
       <c r="D252" t="n">
-        <v>900119</v>
+        <v>302451</v>
       </c>
       <c r="E252" t="inlineStr">
         <is>
@@ -14646,10 +14967,10 @@
         </is>
       </c>
       <c r="C253" t="n">
-        <v>900120</v>
+        <v>900117</v>
       </c>
       <c r="D253" t="n">
-        <v>900121</v>
+        <v>300101</v>
       </c>
       <c r="E253" t="inlineStr">
         <is>
@@ -14667,12 +14988,369 @@
         </is>
       </c>
       <c r="C254" t="n">
+        <v>900119</v>
+      </c>
+      <c r="D254" t="n">
+        <v>900120</v>
+      </c>
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>MANUAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="n">
+        <v>254</v>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>BEAM_Y</t>
+        </is>
+      </c>
+      <c r="C255" t="n">
+        <v>900028</v>
+      </c>
+      <c r="D255" t="n">
+        <v>900121</v>
+      </c>
+      <c r="E255" t="inlineStr">
+        <is>
+          <t>MANUAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="n">
+        <v>255</v>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>BEAM_Y</t>
+        </is>
+      </c>
+      <c r="C256" t="n">
         <v>900122</v>
       </c>
-      <c r="D254" t="n">
+      <c r="D256" t="n">
         <v>900123</v>
       </c>
-      <c r="E254" t="inlineStr">
+      <c r="E256" t="inlineStr">
+        <is>
+          <t>MANUAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="n">
+        <v>256</v>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>BEAM_Y</t>
+        </is>
+      </c>
+      <c r="C257" t="n">
+        <v>900118</v>
+      </c>
+      <c r="D257" t="n">
+        <v>900122</v>
+      </c>
+      <c r="E257" t="inlineStr">
+        <is>
+          <t>MANUAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="n">
+        <v>257</v>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>BEAM_Y</t>
+        </is>
+      </c>
+      <c r="C258" t="n">
+        <v>900124</v>
+      </c>
+      <c r="D258" t="n">
+        <v>900125</v>
+      </c>
+      <c r="E258" t="inlineStr">
+        <is>
+          <t>MANUAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="n">
+        <v>258</v>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>BEAM_X</t>
+        </is>
+      </c>
+      <c r="C259" t="n">
+        <v>400001</v>
+      </c>
+      <c r="D259" t="n">
+        <v>400451</v>
+      </c>
+      <c r="E259" t="inlineStr">
+        <is>
+          <t>MANUAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="n">
+        <v>259</v>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>BEAM_X</t>
+        </is>
+      </c>
+      <c r="C260" t="n">
+        <v>401001</v>
+      </c>
+      <c r="D260" t="n">
+        <v>401451</v>
+      </c>
+      <c r="E260" t="inlineStr">
+        <is>
+          <t>MANUAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="n">
+        <v>260</v>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>BEAM_X</t>
+        </is>
+      </c>
+      <c r="C261" t="n">
+        <v>402001</v>
+      </c>
+      <c r="D261" t="n">
+        <v>402451</v>
+      </c>
+      <c r="E261" t="inlineStr">
+        <is>
+          <t>MANUAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="n">
+        <v>261</v>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>BEAM_Y</t>
+        </is>
+      </c>
+      <c r="C262" t="n">
+        <v>400001</v>
+      </c>
+      <c r="D262" t="n">
+        <v>402001</v>
+      </c>
+      <c r="E262" t="inlineStr">
+        <is>
+          <t>MANUAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="n">
+        <v>262</v>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>BEAM_Y</t>
+        </is>
+      </c>
+      <c r="C263" t="n">
+        <v>400101</v>
+      </c>
+      <c r="D263" t="n">
+        <v>402101</v>
+      </c>
+      <c r="E263" t="inlineStr">
+        <is>
+          <t>MANUAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="n">
+        <v>263</v>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>BEAM_Y</t>
+        </is>
+      </c>
+      <c r="C264" t="n">
+        <v>400201</v>
+      </c>
+      <c r="D264" t="n">
+        <v>402201</v>
+      </c>
+      <c r="E264" t="inlineStr">
+        <is>
+          <t>MANUAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="n">
+        <v>264</v>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>BEAM_Y</t>
+        </is>
+      </c>
+      <c r="C265" t="n">
+        <v>400301</v>
+      </c>
+      <c r="D265" t="n">
+        <v>402301</v>
+      </c>
+      <c r="E265" t="inlineStr">
+        <is>
+          <t>MANUAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="n">
+        <v>265</v>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>BEAM_Y</t>
+        </is>
+      </c>
+      <c r="C266" t="n">
+        <v>400401</v>
+      </c>
+      <c r="D266" t="n">
+        <v>402401</v>
+      </c>
+      <c r="E266" t="inlineStr">
+        <is>
+          <t>MANUAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="n">
+        <v>266</v>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>BEAM_Y</t>
+        </is>
+      </c>
+      <c r="C267" t="n">
+        <v>400451</v>
+      </c>
+      <c r="D267" t="n">
+        <v>402451</v>
+      </c>
+      <c r="E267" t="inlineStr">
+        <is>
+          <t>MANUAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="n">
+        <v>267</v>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>BEAM_Y</t>
+        </is>
+      </c>
+      <c r="C268" t="n">
+        <v>900126</v>
+      </c>
+      <c r="D268" t="n">
+        <v>900127</v>
+      </c>
+      <c r="E268" t="inlineStr">
+        <is>
+          <t>MANUAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="n">
+        <v>268</v>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>BEAM_Y</t>
+        </is>
+      </c>
+      <c r="C269" t="n">
+        <v>900128</v>
+      </c>
+      <c r="D269" t="n">
+        <v>900129</v>
+      </c>
+      <c r="E269" t="inlineStr">
+        <is>
+          <t>MANUAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="n">
+        <v>269</v>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>BEAM_Y</t>
+        </is>
+      </c>
+      <c r="C270" t="n">
+        <v>900130</v>
+      </c>
+      <c r="D270" t="n">
+        <v>900131</v>
+      </c>
+      <c r="E270" t="inlineStr">
+        <is>
+          <t>MANUAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="n">
+        <v>270</v>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>BEAM_Y</t>
+        </is>
+      </c>
+      <c r="C271" t="n">
+        <v>900132</v>
+      </c>
+      <c r="D271" t="n">
+        <v>900133</v>
+      </c>
+      <c r="E271" t="inlineStr">
         <is>
           <t>MANUAL</t>
         </is>
@@ -14689,6 +15367,426 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>nodo_1</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>nodo_2</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>nodo_3</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>nodo_4</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>z_m</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>espesor_m</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>estado</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="B2" t="n">
+        <v>900017</v>
+      </c>
+      <c r="C2" t="n">
+        <v>900018</v>
+      </c>
+      <c r="D2" t="n">
+        <v>900023</v>
+      </c>
+      <c r="E2" t="n">
+        <v>200101</v>
+      </c>
+      <c r="F2" t="n">
+        <v>7.92</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>MANUAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1000001</v>
+      </c>
+      <c r="B3" t="n">
+        <v>900027</v>
+      </c>
+      <c r="C3" t="n">
+        <v>900029</v>
+      </c>
+      <c r="D3" t="n">
+        <v>900028</v>
+      </c>
+      <c r="E3" t="n">
+        <v>300201</v>
+      </c>
+      <c r="F3" t="n">
+        <v>11.88</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>MANUAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>1000002</v>
+      </c>
+      <c r="B4" t="n">
+        <v>900029</v>
+      </c>
+      <c r="C4" t="n">
+        <v>900030</v>
+      </c>
+      <c r="D4" t="n">
+        <v>300301</v>
+      </c>
+      <c r="E4" t="n">
+        <v>900028</v>
+      </c>
+      <c r="F4" t="n">
+        <v>11.88</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>MANUAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>1000003</v>
+      </c>
+      <c r="B5" t="n">
+        <v>900031</v>
+      </c>
+      <c r="C5" t="n">
+        <v>900033</v>
+      </c>
+      <c r="D5" t="n">
+        <v>900032</v>
+      </c>
+      <c r="E5" t="n">
+        <v>400101</v>
+      </c>
+      <c r="F5" t="n">
+        <v>15.84</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>MANUAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>1000004</v>
+      </c>
+      <c r="B6" t="n">
+        <v>400451</v>
+      </c>
+      <c r="C6" t="n">
+        <v>400501</v>
+      </c>
+      <c r="D6" t="n">
+        <v>401501</v>
+      </c>
+      <c r="E6" t="n">
+        <v>401451</v>
+      </c>
+      <c r="F6" t="n">
+        <v>15.84</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>MANUAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>1000005</v>
+      </c>
+      <c r="B7" t="n">
+        <v>401451</v>
+      </c>
+      <c r="C7" t="n">
+        <v>401501</v>
+      </c>
+      <c r="D7" t="n">
+        <v>402501</v>
+      </c>
+      <c r="E7" t="n">
+        <v>402451</v>
+      </c>
+      <c r="F7" t="n">
+        <v>15.84</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>MANUAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>1000006</v>
+      </c>
+      <c r="B8" t="n">
+        <v>900100</v>
+      </c>
+      <c r="C8" t="n">
+        <v>900109</v>
+      </c>
+      <c r="D8" t="n">
+        <v>900110</v>
+      </c>
+      <c r="E8" t="n">
+        <v>900103</v>
+      </c>
+      <c r="F8" t="n">
+        <v>19.8</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>MANUAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>1000007</v>
+      </c>
+      <c r="B9" t="n">
+        <v>900047</v>
+      </c>
+      <c r="C9" t="n">
+        <v>900048</v>
+      </c>
+      <c r="D9" t="n">
+        <v>500301</v>
+      </c>
+      <c r="E9" t="n">
+        <v>500201</v>
+      </c>
+      <c r="F9" t="n">
+        <v>19.8</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>MANUAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>1000008</v>
+      </c>
+      <c r="B10" t="n">
+        <v>900009</v>
+      </c>
+      <c r="C10" t="n">
+        <v>100451</v>
+      </c>
+      <c r="D10" t="n">
+        <v>102451</v>
+      </c>
+      <c r="E10" t="n">
+        <v>900010</v>
+      </c>
+      <c r="F10" t="n">
+        <v>3.96</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>MANUAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>1000009</v>
+      </c>
+      <c r="B11" t="n">
+        <v>900058</v>
+      </c>
+      <c r="C11" t="n">
+        <v>200451</v>
+      </c>
+      <c r="D11" t="n">
+        <v>202451</v>
+      </c>
+      <c r="E11" t="n">
+        <v>900059</v>
+      </c>
+      <c r="F11" t="n">
+        <v>7.92</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>MANUAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>1000010</v>
+      </c>
+      <c r="B12" t="n">
+        <v>900075</v>
+      </c>
+      <c r="C12" t="n">
+        <v>300451</v>
+      </c>
+      <c r="D12" t="n">
+        <v>302451</v>
+      </c>
+      <c r="E12" t="n">
+        <v>900076</v>
+      </c>
+      <c r="F12" t="n">
+        <v>11.88</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>MANUAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>1000011</v>
+      </c>
+      <c r="B13" t="n">
+        <v>900092</v>
+      </c>
+      <c r="C13" t="n">
+        <v>400451</v>
+      </c>
+      <c r="D13" t="n">
+        <v>402451</v>
+      </c>
+      <c r="E13" t="n">
+        <v>900093</v>
+      </c>
+      <c r="F13" t="n">
+        <v>15.84</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>MANUAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>1000012</v>
+      </c>
+      <c r="B14" t="n">
+        <v>900109</v>
+      </c>
+      <c r="C14" t="n">
+        <v>500451</v>
+      </c>
+      <c r="D14" t="n">
+        <v>502451</v>
+      </c>
+      <c r="E14" t="n">
+        <v>900110</v>
+      </c>
+      <c r="F14" t="n">
+        <v>19.8</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>MANUAL</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:B6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
@@ -14760,7 +15858,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Solo vigas y columnas; sin losas, muros ni fundaciones</t>
+          <t>Vigas, columnas, muros y losas cerradas por vigas; sin fundaciones</t>
         </is>
       </c>
     </row>

</xml_diff>